<commit_message>
feat(conf-abstracts): ingest SI2022 Valencia programme (89 talks) + matrix update
SI2022 detailed programme (8pp schedule, clean native text, no OCR): 'Presenter:
Title' talks under 'Session N:' headers -> 89 talks, all elasmo (schedule, no
bodies). Matrix: SI2022 Valencia -> Ingested; EEA2013 Plymouth -> Digital
(abstract book held locally). DB 9,792 records / 3,174 elasmo.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -2742,9 +2742,9 @@
           <t>Albuquerque, NM; Hardcopy</t>
         </is>
       </c>
-      <c r="D99" s="13" t="inlineStr">
-        <is>
-          <t>Plymouth; Hardcopy</t>
+      <c r="D99" s="18" t="inlineStr">
+        <is>
+          <t>Plymouth; Digital</t>
         </is>
       </c>
       <c r="E99" s="12" t="inlineStr"/>
@@ -2974,9 +2974,9 @@
           <t>?; Pending (Brit)</t>
         </is>
       </c>
-      <c r="F108" s="18" t="inlineStr">
-        <is>
-          <t>Valencia; Digital</t>
+      <c r="F108" s="15" t="inlineStr">
+        <is>
+          <t>Valencia; Ingested</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>89</v>
       </c>
     </row>
     <row r="35">
@@ -3968,7 +3968,7 @@
         <v>99</v>
       </c>
       <c r="G39" s="1" t="n">
-        <v>1428</v>
+        <v>1517</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(conf-abstracts): EEA 2015 abstract book held (Digital); 2017/2023 programmes held
EEA History folder holds EEA 2013+2015 abstract books, 2017/2021/2023
programmes, and AES presentation extracts (2015/16/17/19). Matrix updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -2794,9 +2794,9 @@
           <t>Reno, NV (123); Ingested</t>
         </is>
       </c>
-      <c r="D101" s="13" t="inlineStr">
-        <is>
-          <t>Peniche; Hardcopy</t>
+      <c r="D101" s="18" t="inlineStr">
+        <is>
+          <t>Peniche; Digital</t>
         </is>
       </c>
       <c r="E101" s="12" t="inlineStr"/>
@@ -2842,9 +2842,9 @@
           <t>Austin, TX; Hardcopy</t>
         </is>
       </c>
-      <c r="D103" s="13" t="inlineStr">
-        <is>
-          <t>Amsterdam; Hardcopy</t>
+      <c r="D103" s="18" t="inlineStr">
+        <is>
+          <t>Amsterdam; Digital</t>
         </is>
       </c>
       <c r="E103" s="12" t="inlineStr"/>

</xml_diff>

<commit_message>
docs(conf-abstracts): 2017/2019 grid program books held but not ingestable
AES 2017/2019 talk detail is in interleaved multi-column grids; number-anchored
extraction yields garbage. 2015/2016 AES 'SharkOnly' lists are redundant (full
abstract books already ingested: 545/1040 with bodies). Matrix: 2017/2019 ->
Digital (held, not ingested). Recommend Carylanne's 2017/2019 abstract books.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -2832,14 +2832,14 @@
       <c r="A103" s="10" t="n">
         <v>2017</v>
       </c>
-      <c r="B103" s="13" t="inlineStr">
-        <is>
-          <t>Austin, TX; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C103" s="13" t="inlineStr">
-        <is>
-          <t>Austin, TX; Hardcopy</t>
+      <c r="B103" s="18" t="inlineStr">
+        <is>
+          <t>Austin, TX; Digital</t>
+        </is>
+      </c>
+      <c r="C103" s="18" t="inlineStr">
+        <is>
+          <t>Austin, TX; Digital</t>
         </is>
       </c>
       <c r="D103" s="18" t="inlineStr">
@@ -2884,14 +2884,14 @@
       <c r="A105" s="10" t="n">
         <v>2019</v>
       </c>
-      <c r="B105" s="13" t="inlineStr">
-        <is>
-          <t>Snowbird, UT; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C105" s="13" t="inlineStr">
-        <is>
-          <t>Snowbird, UT; Hardcopy</t>
+      <c r="B105" s="18" t="inlineStr">
+        <is>
+          <t>Snowbird, UT; Digital</t>
+        </is>
+      </c>
+      <c r="C105" s="18" t="inlineStr">
+        <is>
+          <t>Snowbird, UT; Digital</t>
         </is>
       </c>
       <c r="D105" s="13" t="inlineStr">

</xml_diff>

<commit_message>
fix(conf-abstracts): faithful status reporting in coverage matrix
Add 'Programme' status (tan): a digital programme/schedule PDF is held but it is
NOT full abstracts — the abstract book is still needed. Distinguishes 2017/2019
(grid programme, abstract book needed from Carylanne) and EEA programmes from
'Digital' (ingestable abstract book held, e.g. EEA 2013/2015). Every cell now
carries an action note: what we hold + what's still needed + who to ask.
'Pending' = available from a contact, not yet obtained (Cat/Brit).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -42,7 +42,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +57,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F6B26B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9CB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -116,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,7 +131,8 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,16 +145,19 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -936,7 +945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -968,7 +977,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>No known source</t>
+          <t>No known source anywhere</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -989,12 +998,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Digital</t>
+          <t>Programme</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Digital PDF exists but not yet ingested</t>
+          <t>Digital PROGRAMME/schedule held, but NOT full abstracts — the abstract book is still needed (see note)</t>
         </is>
       </c>
       <c r="C4" s="4" t="n"/>
@@ -1002,12 +1011,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>OCR</t>
+          <t>Digital</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OCR'd &amp; ingested but low-confidence (needs_review) — old degraded scans</t>
+          <t>Digital ABSTRACT BOOK held &amp; ingestable, not yet ingested</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
@@ -1015,12 +1024,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Schedule</t>
+          <t>OCR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Program book ingested: titles/authors/type, NO abstract bodies</t>
+          <t>Full abstracts ingested but from degraded scans (needs_review) — flatbed re-scan planned</t>
         </is>
       </c>
       <c r="C6" s="6" t="n"/>
@@ -1028,12 +1037,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ingested</t>
+          <t>Schedule</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Full abstracts ingested into the DB</t>
+          <t>Programme ingested: titles/authors/type, NO abstract bodies</t>
         </is>
       </c>
       <c r="C7" s="7" t="n"/>
@@ -1041,84 +1050,97 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Ingested</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Full abstracts ingested into the DB</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Being collated by an external contact (OCS: Brit Finucci)</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Available from an external contact, not yet obtained (EEA: Cat; OCS: Brit)</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>NOTES:</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>- 'ASIH/JMIH' = the American joint meeting (ASIH pre-1997, JMIH from 1997). ASIH/JMIH/HL/SSAR/NIA share one source book, collapsed to this column to remove duplicates.</t>
+          <t>NOTES:</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>- 'AES' (American Elasmobranch Society, founded 1983) kept separate — cell shows elasmo-abstract count where ingested. Pre-1983 = no conference (blank).</t>
+          <t>- 'ASIH/JMIH' = the American joint meeting (ASIH pre-1997, JMIH from 1997). ASIH/JMIH/HL/SSAR/NIA share one source book, collapsed to this column to remove duplicates.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>- Host cities 1916-2025 from github.com/SimonDedman/AESconfLocations; 2026 = New Orleans.</t>
+          <t>- 'AES' (American Elasmobranch Society, founded 1983) kept separate — cell shows elasmo-abstract count where ingested. Pre-1983 = no conference (blank).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>- 'OCR' = degraded 1997-2004 JMIH phone-photo scans (all needs_review); Carylanne's flatbed re-scans will upgrade these.</t>
+          <t>- Host cities 1916-2025 from github.com/SimonDedman/AESconfLocations; 2026 = New Orleans.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>- No abstracts collected pre-1992 (Carylanne's archive starts 1992) → 1916-1991 show host city but 'Missing'.</t>
+          <t>- 'OCR' = degraded 1997-2004 JMIH phone-photo scans (all needs_review); Carylanne's flatbed re-scans will upgrade these.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>- EEA 2010-2026 from Cat Gordon (Shark Trust); pre-2010 in Ali's archive. EEA not yet ingested. SI2022 Valencia PDF received (Digital).</t>
+          <t>- No abstracts collected pre-1992 (Carylanne's archive starts 1992) → 1916-1991 show host city but 'Missing'.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>- OCS (Oceania Chondrichthyan Soc, ~2011+, biennial): Brit Finucci collating, pending council — years/locations TBC.</t>
+          <t>- EEA 2010-2026 from Cat Gordon (Shark Trust); pre-2010 in Ali's archive. EEA not yet ingested. SI2022 Valencia PDF received (Digital).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>- Blank/unshaded cell = no conference that year for that series.</t>
+          <t>- OCS (Oceania Chondrichthyan Soc, ~2011+, biennial): Brit Finucci collating, pending council — years/locations TBC.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
+        <is>
+          <t>- Blank/unshaded cell = no conference that year for that series.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>- Per-society counts &amp; trends: see the Dashboard tab.</t>
         </is>
@@ -1139,1942 +1161,1942 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>ASIH/JMIH</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>AES</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>EEA</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>OCS</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="n">
+      <c r="A2" s="11" t="n">
         <v>1916</v>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>New York, NY; Missing</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr"/>
-      <c r="D2" s="12" t="inlineStr"/>
-      <c r="E2" s="12" t="inlineStr"/>
-      <c r="F2" s="12" t="inlineStr"/>
+      <c r="C2" s="13" t="inlineStr"/>
+      <c r="D2" s="13" t="inlineStr"/>
+      <c r="E2" s="13" t="inlineStr"/>
+      <c r="F2" s="13" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="n">
+      <c r="A3" s="11" t="n">
         <v>1917</v>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Cambridge, MA; Missing</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr"/>
-      <c r="D3" s="12" t="inlineStr"/>
-      <c r="E3" s="12" t="inlineStr"/>
-      <c r="F3" s="12" t="inlineStr"/>
+      <c r="C3" s="13" t="inlineStr"/>
+      <c r="D3" s="13" t="inlineStr"/>
+      <c r="E3" s="13" t="inlineStr"/>
+      <c r="F3" s="13" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="n">
+      <c r="A4" s="11" t="n">
         <v>1918</v>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Brooklyn, NY; Missing</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr"/>
-      <c r="D4" s="12" t="inlineStr"/>
-      <c r="E4" s="12" t="inlineStr"/>
-      <c r="F4" s="12" t="inlineStr"/>
+      <c r="C4" s="13" t="inlineStr"/>
+      <c r="D4" s="13" t="inlineStr"/>
+      <c r="E4" s="13" t="inlineStr"/>
+      <c r="F4" s="13" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="n">
+      <c r="A5" s="11" t="n">
         <v>1919</v>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>?; Missing</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr"/>
-      <c r="D5" s="12" t="inlineStr"/>
-      <c r="E5" s="12" t="inlineStr"/>
-      <c r="F5" s="12" t="inlineStr"/>
+      <c r="C5" s="13" t="inlineStr"/>
+      <c r="D5" s="13" t="inlineStr"/>
+      <c r="E5" s="13" t="inlineStr"/>
+      <c r="F5" s="13" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="n">
+      <c r="A6" s="11" t="n">
         <v>1920</v>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Washington, DC; Missing</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr"/>
-      <c r="D6" s="12" t="inlineStr"/>
-      <c r="E6" s="12" t="inlineStr"/>
-      <c r="F6" s="12" t="inlineStr"/>
+      <c r="C6" s="13" t="inlineStr"/>
+      <c r="D6" s="13" t="inlineStr"/>
+      <c r="E6" s="13" t="inlineStr"/>
+      <c r="F6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="n">
+      <c r="A7" s="11" t="n">
         <v>1921</v>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Philadelphia, PA; Missing</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr"/>
-      <c r="D7" s="12" t="inlineStr"/>
-      <c r="E7" s="12" t="inlineStr"/>
-      <c r="F7" s="12" t="inlineStr"/>
+      <c r="C7" s="13" t="inlineStr"/>
+      <c r="D7" s="13" t="inlineStr"/>
+      <c r="E7" s="13" t="inlineStr"/>
+      <c r="F7" s="13" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="n">
+      <c r="A8" s="11" t="n">
         <v>1922</v>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Chicago, IL; Missing</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr"/>
-      <c r="D8" s="12" t="inlineStr"/>
-      <c r="E8" s="12" t="inlineStr"/>
-      <c r="F8" s="12" t="inlineStr"/>
+      <c r="C8" s="13" t="inlineStr"/>
+      <c r="D8" s="13" t="inlineStr"/>
+      <c r="E8" s="13" t="inlineStr"/>
+      <c r="F8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n">
+      <c r="A9" s="11" t="n">
         <v>1923</v>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Cambridge, MA; Missing</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr"/>
-      <c r="D9" s="12" t="inlineStr"/>
-      <c r="E9" s="12" t="inlineStr"/>
-      <c r="F9" s="12" t="inlineStr"/>
+      <c r="C9" s="13" t="inlineStr"/>
+      <c r="D9" s="13" t="inlineStr"/>
+      <c r="E9" s="13" t="inlineStr"/>
+      <c r="F9" s="13" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="n">
+      <c r="A10" s="11" t="n">
         <v>1924</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Northhampton, MA; Missing</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr"/>
-      <c r="D10" s="12" t="inlineStr"/>
-      <c r="E10" s="12" t="inlineStr"/>
-      <c r="F10" s="12" t="inlineStr"/>
+      <c r="C10" s="13" t="inlineStr"/>
+      <c r="D10" s="13" t="inlineStr"/>
+      <c r="E10" s="13" t="inlineStr"/>
+      <c r="F10" s="13" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n">
+      <c r="A11" s="11" t="n">
         <v>1925</v>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>?; Missing</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr"/>
-      <c r="D11" s="12" t="inlineStr"/>
-      <c r="E11" s="12" t="inlineStr"/>
-      <c r="F11" s="12" t="inlineStr"/>
+      <c r="C11" s="13" t="inlineStr"/>
+      <c r="D11" s="13" t="inlineStr"/>
+      <c r="E11" s="13" t="inlineStr"/>
+      <c r="F11" s="13" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n">
+      <c r="A12" s="11" t="n">
         <v>1926</v>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Philadelphia, PA; Missing</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr"/>
-      <c r="D12" s="12" t="inlineStr"/>
-      <c r="E12" s="12" t="inlineStr"/>
-      <c r="F12" s="12" t="inlineStr"/>
+      <c r="C12" s="13" t="inlineStr"/>
+      <c r="D12" s="13" t="inlineStr"/>
+      <c r="E12" s="13" t="inlineStr"/>
+      <c r="F12" s="13" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n">
+      <c r="A13" s="11" t="n">
         <v>1927</v>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Philadelphia, PA; Missing</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr"/>
-      <c r="D13" s="12" t="inlineStr"/>
-      <c r="E13" s="12" t="inlineStr"/>
-      <c r="F13" s="12" t="inlineStr"/>
+      <c r="C13" s="13" t="inlineStr"/>
+      <c r="D13" s="13" t="inlineStr"/>
+      <c r="E13" s="13" t="inlineStr"/>
+      <c r="F13" s="13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n">
+      <c r="A14" s="11" t="n">
         <v>1928</v>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Washington, DC; Missing</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr"/>
-      <c r="D14" s="12" t="inlineStr"/>
-      <c r="E14" s="12" t="inlineStr"/>
-      <c r="F14" s="12" t="inlineStr"/>
+      <c r="C14" s="13" t="inlineStr"/>
+      <c r="D14" s="13" t="inlineStr"/>
+      <c r="E14" s="13" t="inlineStr"/>
+      <c r="F14" s="13" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="n">
+      <c r="A15" s="11" t="n">
         <v>1929</v>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Ann Arbor, MI; Missing</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr"/>
-      <c r="D15" s="12" t="inlineStr"/>
-      <c r="E15" s="12" t="inlineStr"/>
-      <c r="F15" s="12" t="inlineStr"/>
+      <c r="C15" s="13" t="inlineStr"/>
+      <c r="D15" s="13" t="inlineStr"/>
+      <c r="E15" s="13" t="inlineStr"/>
+      <c r="F15" s="13" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n">
+      <c r="A16" s="11" t="n">
         <v>1930</v>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>New York, NY; Missing</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr"/>
-      <c r="D16" s="12" t="inlineStr"/>
-      <c r="E16" s="12" t="inlineStr"/>
-      <c r="F16" s="12" t="inlineStr"/>
+      <c r="C16" s="13" t="inlineStr"/>
+      <c r="D16" s="13" t="inlineStr"/>
+      <c r="E16" s="13" t="inlineStr"/>
+      <c r="F16" s="13" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="n">
+      <c r="A17" s="11" t="n">
         <v>1931</v>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Philadelphia, PA; Missing</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr"/>
-      <c r="D17" s="12" t="inlineStr"/>
-      <c r="E17" s="12" t="inlineStr"/>
-      <c r="F17" s="12" t="inlineStr"/>
+      <c r="C17" s="13" t="inlineStr"/>
+      <c r="D17" s="13" t="inlineStr"/>
+      <c r="E17" s="13" t="inlineStr"/>
+      <c r="F17" s="13" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n">
+      <c r="A18" s="11" t="n">
         <v>1932</v>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Washington, DC; Missing</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr"/>
-      <c r="D18" s="12" t="inlineStr"/>
-      <c r="E18" s="12" t="inlineStr"/>
-      <c r="F18" s="12" t="inlineStr"/>
+      <c r="C18" s="13" t="inlineStr"/>
+      <c r="D18" s="13" t="inlineStr"/>
+      <c r="E18" s="13" t="inlineStr"/>
+      <c r="F18" s="13" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="n">
+      <c r="A19" s="11" t="n">
         <v>1933</v>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Cambridge, MA; Missing</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr"/>
-      <c r="D19" s="12" t="inlineStr"/>
-      <c r="E19" s="12" t="inlineStr"/>
-      <c r="F19" s="12" t="inlineStr"/>
+      <c r="C19" s="13" t="inlineStr"/>
+      <c r="D19" s="13" t="inlineStr"/>
+      <c r="E19" s="13" t="inlineStr"/>
+      <c r="F19" s="13" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n">
+      <c r="A20" s="11" t="n">
         <v>1934</v>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>New York, NY; Missing</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr"/>
-      <c r="D20" s="12" t="inlineStr"/>
-      <c r="E20" s="12" t="inlineStr"/>
-      <c r="F20" s="12" t="inlineStr"/>
+      <c r="C20" s="13" t="inlineStr"/>
+      <c r="D20" s="13" t="inlineStr"/>
+      <c r="E20" s="13" t="inlineStr"/>
+      <c r="F20" s="13" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="n">
+      <c r="A21" s="11" t="n">
         <v>1935</v>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Pittsburgh, PA; Missing</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr"/>
-      <c r="D21" s="12" t="inlineStr"/>
-      <c r="E21" s="12" t="inlineStr"/>
-      <c r="F21" s="12" t="inlineStr"/>
+      <c r="C21" s="13" t="inlineStr"/>
+      <c r="D21" s="13" t="inlineStr"/>
+      <c r="E21" s="13" t="inlineStr"/>
+      <c r="F21" s="13" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="n">
+      <c r="A22" s="11" t="n">
         <v>1936</v>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Ann Arbor, MI; Missing</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr"/>
-      <c r="D22" s="12" t="inlineStr"/>
-      <c r="E22" s="12" t="inlineStr"/>
-      <c r="F22" s="12" t="inlineStr"/>
+      <c r="C22" s="13" t="inlineStr"/>
+      <c r="D22" s="13" t="inlineStr"/>
+      <c r="E22" s="13" t="inlineStr"/>
+      <c r="F22" s="13" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="n">
+      <c r="A23" s="11" t="n">
         <v>1937</v>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Washington, DC; Missing</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr"/>
-      <c r="D23" s="12" t="inlineStr"/>
-      <c r="E23" s="12" t="inlineStr"/>
-      <c r="F23" s="12" t="inlineStr"/>
+      <c r="C23" s="13" t="inlineStr"/>
+      <c r="D23" s="13" t="inlineStr"/>
+      <c r="E23" s="13" t="inlineStr"/>
+      <c r="F23" s="13" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="n">
+      <c r="A24" s="11" t="n">
         <v>1938</v>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Berkeley, CA; Missing</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr"/>
-      <c r="D24" s="12" t="inlineStr"/>
-      <c r="E24" s="12" t="inlineStr"/>
-      <c r="F24" s="12" t="inlineStr"/>
+      <c r="C24" s="13" t="inlineStr"/>
+      <c r="D24" s="13" t="inlineStr"/>
+      <c r="E24" s="13" t="inlineStr"/>
+      <c r="F24" s="13" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="n">
+      <c r="A25" s="11" t="n">
         <v>1939</v>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Chicago, IL; Missing</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr"/>
-      <c r="D25" s="12" t="inlineStr"/>
-      <c r="E25" s="12" t="inlineStr"/>
-      <c r="F25" s="12" t="inlineStr"/>
+      <c r="C25" s="13" t="inlineStr"/>
+      <c r="D25" s="13" t="inlineStr"/>
+      <c r="E25" s="13" t="inlineStr"/>
+      <c r="F25" s="13" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="n">
+      <c r="A26" s="11" t="n">
         <v>1940</v>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>Toronto, ON; Missing</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr"/>
-      <c r="D26" s="12" t="inlineStr"/>
-      <c r="E26" s="12" t="inlineStr"/>
-      <c r="F26" s="12" t="inlineStr"/>
+      <c r="C26" s="13" t="inlineStr"/>
+      <c r="D26" s="13" t="inlineStr"/>
+      <c r="E26" s="13" t="inlineStr"/>
+      <c r="F26" s="13" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="n">
+      <c r="A27" s="11" t="n">
         <v>1941</v>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>Gainesville, FL; Missing</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr"/>
-      <c r="D27" s="12" t="inlineStr"/>
-      <c r="E27" s="12" t="inlineStr"/>
-      <c r="F27" s="12" t="inlineStr"/>
+      <c r="C27" s="13" t="inlineStr"/>
+      <c r="D27" s="13" t="inlineStr"/>
+      <c r="E27" s="13" t="inlineStr"/>
+      <c r="F27" s="13" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="n">
+      <c r="A28" s="11" t="n">
         <v>1942</v>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>New York, NY; Missing</t>
         </is>
       </c>
-      <c r="C28" s="12" t="inlineStr"/>
-      <c r="D28" s="12" t="inlineStr"/>
-      <c r="E28" s="12" t="inlineStr"/>
-      <c r="F28" s="12" t="inlineStr"/>
+      <c r="C28" s="13" t="inlineStr"/>
+      <c r="D28" s="13" t="inlineStr"/>
+      <c r="E28" s="13" t="inlineStr"/>
+      <c r="F28" s="13" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="n">
+      <c r="A29" s="11" t="n">
         <v>1943</v>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>?; Missing</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr"/>
-      <c r="D29" s="12" t="inlineStr"/>
-      <c r="E29" s="12" t="inlineStr"/>
-      <c r="F29" s="12" t="inlineStr"/>
+      <c r="C29" s="13" t="inlineStr"/>
+      <c r="D29" s="13" t="inlineStr"/>
+      <c r="E29" s="13" t="inlineStr"/>
+      <c r="F29" s="13" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="n">
+      <c r="A30" s="11" t="n">
         <v>1944</v>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>?; Missing</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr"/>
-      <c r="D30" s="12" t="inlineStr"/>
-      <c r="E30" s="12" t="inlineStr"/>
-      <c r="F30" s="12" t="inlineStr"/>
+      <c r="C30" s="13" t="inlineStr"/>
+      <c r="D30" s="13" t="inlineStr"/>
+      <c r="E30" s="13" t="inlineStr"/>
+      <c r="F30" s="13" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="n">
+      <c r="A31" s="11" t="n">
         <v>1945</v>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>?; Missing</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr"/>
-      <c r="D31" s="12" t="inlineStr"/>
-      <c r="E31" s="12" t="inlineStr"/>
-      <c r="F31" s="12" t="inlineStr"/>
+      <c r="C31" s="13" t="inlineStr"/>
+      <c r="D31" s="13" t="inlineStr"/>
+      <c r="E31" s="13" t="inlineStr"/>
+      <c r="F31" s="13" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="n">
+      <c r="A32" s="11" t="n">
         <v>1946</v>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>Pittsburgh, PA; Missing</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr"/>
-      <c r="D32" s="12" t="inlineStr"/>
-      <c r="E32" s="12" t="inlineStr"/>
-      <c r="F32" s="12" t="inlineStr"/>
+      <c r="C32" s="13" t="inlineStr"/>
+      <c r="D32" s="13" t="inlineStr"/>
+      <c r="E32" s="13" t="inlineStr"/>
+      <c r="F32" s="13" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="n">
+      <c r="A33" s="11" t="n">
         <v>1947</v>
       </c>
-      <c r="B33" s="11" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Higgins Lake, MI; Missing</t>
         </is>
       </c>
-      <c r="C33" s="12" t="inlineStr"/>
-      <c r="D33" s="12" t="inlineStr"/>
-      <c r="E33" s="12" t="inlineStr"/>
-      <c r="F33" s="12" t="inlineStr"/>
+      <c r="C33" s="13" t="inlineStr"/>
+      <c r="D33" s="13" t="inlineStr"/>
+      <c r="E33" s="13" t="inlineStr"/>
+      <c r="F33" s="13" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="n">
+      <c r="A34" s="11" t="n">
         <v>1948</v>
       </c>
-      <c r="B34" s="11" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>New Orleans, LA; Missing</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr"/>
-      <c r="D34" s="12" t="inlineStr"/>
-      <c r="E34" s="12" t="inlineStr"/>
-      <c r="F34" s="12" t="inlineStr"/>
+      <c r="C34" s="13" t="inlineStr"/>
+      <c r="D34" s="13" t="inlineStr"/>
+      <c r="E34" s="13" t="inlineStr"/>
+      <c r="F34" s="13" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="n">
+      <c r="A35" s="11" t="n">
         <v>1949</v>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Washington, DC; Missing</t>
         </is>
       </c>
-      <c r="C35" s="12" t="inlineStr"/>
-      <c r="D35" s="12" t="inlineStr"/>
-      <c r="E35" s="12" t="inlineStr"/>
-      <c r="F35" s="12" t="inlineStr"/>
+      <c r="C35" s="13" t="inlineStr"/>
+      <c r="D35" s="13" t="inlineStr"/>
+      <c r="E35" s="13" t="inlineStr"/>
+      <c r="F35" s="13" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="n">
+      <c r="A36" s="11" t="n">
         <v>1950</v>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Salt Lake City, UT; Missing</t>
         </is>
       </c>
-      <c r="C36" s="12" t="inlineStr"/>
-      <c r="D36" s="12" t="inlineStr"/>
-      <c r="E36" s="12" t="inlineStr"/>
-      <c r="F36" s="12" t="inlineStr"/>
+      <c r="C36" s="13" t="inlineStr"/>
+      <c r="D36" s="13" t="inlineStr"/>
+      <c r="E36" s="13" t="inlineStr"/>
+      <c r="F36" s="13" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="n">
+      <c r="A37" s="11" t="n">
         <v>1951</v>
       </c>
-      <c r="B37" s="11" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>Chicago, IL; Missing</t>
         </is>
       </c>
-      <c r="C37" s="12" t="inlineStr"/>
-      <c r="D37" s="12" t="inlineStr"/>
-      <c r="E37" s="12" t="inlineStr"/>
-      <c r="F37" s="12" t="inlineStr"/>
+      <c r="C37" s="13" t="inlineStr"/>
+      <c r="D37" s="13" t="inlineStr"/>
+      <c r="E37" s="13" t="inlineStr"/>
+      <c r="F37" s="13" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="n">
+      <c r="A38" s="11" t="n">
         <v>1952</v>
       </c>
-      <c r="B38" s="11" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>Austin, TX; Missing</t>
         </is>
       </c>
-      <c r="C38" s="12" t="inlineStr"/>
-      <c r="D38" s="12" t="inlineStr"/>
-      <c r="E38" s="12" t="inlineStr"/>
-      <c r="F38" s="12" t="inlineStr"/>
+      <c r="C38" s="13" t="inlineStr"/>
+      <c r="D38" s="13" t="inlineStr"/>
+      <c r="E38" s="13" t="inlineStr"/>
+      <c r="F38" s="13" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="n">
+      <c r="A39" s="11" t="n">
         <v>1953</v>
       </c>
-      <c r="B39" s="11" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>New York, NY; Missing</t>
         </is>
       </c>
-      <c r="C39" s="12" t="inlineStr"/>
-      <c r="D39" s="12" t="inlineStr"/>
-      <c r="E39" s="12" t="inlineStr"/>
-      <c r="F39" s="12" t="inlineStr"/>
+      <c r="C39" s="13" t="inlineStr"/>
+      <c r="D39" s="13" t="inlineStr"/>
+      <c r="E39" s="13" t="inlineStr"/>
+      <c r="F39" s="13" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="n">
+      <c r="A40" s="11" t="n">
         <v>1954</v>
       </c>
-      <c r="B40" s="11" t="inlineStr">
+      <c r="B40" s="12" t="inlineStr">
         <is>
           <t>Gainesville, FL; Missing</t>
         </is>
       </c>
-      <c r="C40" s="12" t="inlineStr"/>
-      <c r="D40" s="12" t="inlineStr"/>
-      <c r="E40" s="12" t="inlineStr"/>
-      <c r="F40" s="12" t="inlineStr"/>
+      <c r="C40" s="13" t="inlineStr"/>
+      <c r="D40" s="13" t="inlineStr"/>
+      <c r="E40" s="13" t="inlineStr"/>
+      <c r="F40" s="13" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="n">
+      <c r="A41" s="11" t="n">
         <v>1955</v>
       </c>
-      <c r="B41" s="11" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
         <is>
           <t>San Francisco, CA; Missing</t>
         </is>
       </c>
-      <c r="C41" s="12" t="inlineStr"/>
-      <c r="D41" s="12" t="inlineStr"/>
-      <c r="E41" s="12" t="inlineStr"/>
-      <c r="F41" s="12" t="inlineStr"/>
+      <c r="C41" s="13" t="inlineStr"/>
+      <c r="D41" s="13" t="inlineStr"/>
+      <c r="E41" s="13" t="inlineStr"/>
+      <c r="F41" s="13" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="10" t="n">
+      <c r="A42" s="11" t="n">
         <v>1956</v>
       </c>
-      <c r="B42" s="11" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
         <is>
           <t>Higgins Lake, MI; Missing</t>
         </is>
       </c>
-      <c r="C42" s="12" t="inlineStr"/>
-      <c r="D42" s="12" t="inlineStr"/>
-      <c r="E42" s="12" t="inlineStr"/>
-      <c r="F42" s="12" t="inlineStr"/>
+      <c r="C42" s="13" t="inlineStr"/>
+      <c r="D42" s="13" t="inlineStr"/>
+      <c r="E42" s="13" t="inlineStr"/>
+      <c r="F42" s="13" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="10" t="n">
+      <c r="A43" s="11" t="n">
         <v>1957</v>
       </c>
-      <c r="B43" s="11" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>New Orleans, LA; Missing</t>
         </is>
       </c>
-      <c r="C43" s="12" t="inlineStr"/>
-      <c r="D43" s="12" t="inlineStr"/>
-      <c r="E43" s="12" t="inlineStr"/>
-      <c r="F43" s="12" t="inlineStr"/>
+      <c r="C43" s="13" t="inlineStr"/>
+      <c r="D43" s="13" t="inlineStr"/>
+      <c r="E43" s="13" t="inlineStr"/>
+      <c r="F43" s="13" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="n">
+      <c r="A44" s="11" t="n">
         <v>1958</v>
       </c>
-      <c r="B44" s="11" t="inlineStr">
+      <c r="B44" s="12" t="inlineStr">
         <is>
           <t>Bloomington, IN; Missing</t>
         </is>
       </c>
-      <c r="C44" s="12" t="inlineStr"/>
-      <c r="D44" s="12" t="inlineStr"/>
-      <c r="E44" s="12" t="inlineStr"/>
-      <c r="F44" s="12" t="inlineStr"/>
+      <c r="C44" s="13" t="inlineStr"/>
+      <c r="D44" s="13" t="inlineStr"/>
+      <c r="E44" s="13" t="inlineStr"/>
+      <c r="F44" s="13" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="10" t="n">
+      <c r="A45" s="11" t="n">
         <v>1959</v>
       </c>
-      <c r="B45" s="11" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t>San Diego, CA; Missing</t>
         </is>
       </c>
-      <c r="C45" s="12" t="inlineStr"/>
-      <c r="D45" s="12" t="inlineStr"/>
-      <c r="E45" s="12" t="inlineStr"/>
-      <c r="F45" s="12" t="inlineStr"/>
+      <c r="C45" s="13" t="inlineStr"/>
+      <c r="D45" s="13" t="inlineStr"/>
+      <c r="E45" s="13" t="inlineStr"/>
+      <c r="F45" s="13" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="10" t="n">
+      <c r="A46" s="11" t="n">
         <v>1960</v>
       </c>
-      <c r="B46" s="11" t="inlineStr">
+      <c r="B46" s="12" t="inlineStr">
         <is>
           <t>Chicago, IL; Missing</t>
         </is>
       </c>
-      <c r="C46" s="12" t="inlineStr"/>
-      <c r="D46" s="12" t="inlineStr"/>
-      <c r="E46" s="12" t="inlineStr"/>
-      <c r="F46" s="12" t="inlineStr"/>
+      <c r="C46" s="13" t="inlineStr"/>
+      <c r="D46" s="13" t="inlineStr"/>
+      <c r="E46" s="13" t="inlineStr"/>
+      <c r="F46" s="13" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="10" t="n">
+      <c r="A47" s="11" t="n">
         <v>1961</v>
       </c>
-      <c r="B47" s="11" t="inlineStr">
+      <c r="B47" s="12" t="inlineStr">
         <is>
           <t>Austin, TX; Missing</t>
         </is>
       </c>
-      <c r="C47" s="12" t="inlineStr"/>
-      <c r="D47" s="12" t="inlineStr"/>
-      <c r="E47" s="12" t="inlineStr"/>
-      <c r="F47" s="12" t="inlineStr"/>
+      <c r="C47" s="13" t="inlineStr"/>
+      <c r="D47" s="13" t="inlineStr"/>
+      <c r="E47" s="13" t="inlineStr"/>
+      <c r="F47" s="13" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="10" t="n">
+      <c r="A48" s="11" t="n">
         <v>1962</v>
       </c>
-      <c r="B48" s="11" t="inlineStr">
+      <c r="B48" s="12" t="inlineStr">
         <is>
           <t>Washington, DC; Missing</t>
         </is>
       </c>
-      <c r="C48" s="12" t="inlineStr"/>
-      <c r="D48" s="12" t="inlineStr"/>
-      <c r="E48" s="12" t="inlineStr"/>
-      <c r="F48" s="12" t="inlineStr"/>
+      <c r="C48" s="13" t="inlineStr"/>
+      <c r="D48" s="13" t="inlineStr"/>
+      <c r="E48" s="13" t="inlineStr"/>
+      <c r="F48" s="13" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="10" t="n">
+      <c r="A49" s="11" t="n">
         <v>1963</v>
       </c>
-      <c r="B49" s="11" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>Vancouver, BC; Missing</t>
         </is>
       </c>
-      <c r="C49" s="12" t="inlineStr"/>
-      <c r="D49" s="12" t="inlineStr"/>
-      <c r="E49" s="12" t="inlineStr"/>
-      <c r="F49" s="12" t="inlineStr"/>
+      <c r="C49" s="13" t="inlineStr"/>
+      <c r="D49" s="13" t="inlineStr"/>
+      <c r="E49" s="13" t="inlineStr"/>
+      <c r="F49" s="13" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="10" t="n">
+      <c r="A50" s="11" t="n">
         <v>1964</v>
       </c>
-      <c r="B50" s="11" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>Morehead City, NC; Missing</t>
         </is>
       </c>
-      <c r="C50" s="12" t="inlineStr"/>
-      <c r="D50" s="12" t="inlineStr"/>
-      <c r="E50" s="12" t="inlineStr"/>
-      <c r="F50" s="12" t="inlineStr"/>
+      <c r="C50" s="13" t="inlineStr"/>
+      <c r="D50" s="13" t="inlineStr"/>
+      <c r="E50" s="13" t="inlineStr"/>
+      <c r="F50" s="13" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="10" t="n">
+      <c r="A51" s="11" t="n">
         <v>1965</v>
       </c>
-      <c r="B51" s="11" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>Lawrence, KS; Missing</t>
         </is>
       </c>
-      <c r="C51" s="12" t="inlineStr"/>
-      <c r="D51" s="12" t="inlineStr"/>
-      <c r="E51" s="12" t="inlineStr"/>
-      <c r="F51" s="12" t="inlineStr"/>
+      <c r="C51" s="13" t="inlineStr"/>
+      <c r="D51" s="13" t="inlineStr"/>
+      <c r="E51" s="13" t="inlineStr"/>
+      <c r="F51" s="13" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="10" t="n">
+      <c r="A52" s="11" t="n">
         <v>1966</v>
       </c>
-      <c r="B52" s="11" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
         <is>
           <t>Miami, FL; Missing</t>
         </is>
       </c>
-      <c r="C52" s="12" t="inlineStr"/>
-      <c r="D52" s="12" t="inlineStr"/>
-      <c r="E52" s="12" t="inlineStr"/>
-      <c r="F52" s="12" t="inlineStr"/>
+      <c r="C52" s="13" t="inlineStr"/>
+      <c r="D52" s="13" t="inlineStr"/>
+      <c r="E52" s="13" t="inlineStr"/>
+      <c r="F52" s="13" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="10" t="n">
+      <c r="A53" s="11" t="n">
         <v>1967</v>
       </c>
-      <c r="B53" s="11" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>San Francisco, CA; Missing</t>
         </is>
       </c>
-      <c r="C53" s="12" t="inlineStr"/>
-      <c r="D53" s="12" t="inlineStr"/>
-      <c r="E53" s="12" t="inlineStr"/>
-      <c r="F53" s="12" t="inlineStr"/>
+      <c r="C53" s="13" t="inlineStr"/>
+      <c r="D53" s="13" t="inlineStr"/>
+      <c r="E53" s="13" t="inlineStr"/>
+      <c r="F53" s="13" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="10" t="n">
+      <c r="A54" s="11" t="n">
         <v>1968</v>
       </c>
-      <c r="B54" s="11" t="inlineStr">
+      <c r="B54" s="12" t="inlineStr">
         <is>
           <t>Ann Arbor, MI; Missing</t>
         </is>
       </c>
-      <c r="C54" s="12" t="inlineStr"/>
-      <c r="D54" s="12" t="inlineStr"/>
-      <c r="E54" s="12" t="inlineStr"/>
-      <c r="F54" s="12" t="inlineStr"/>
+      <c r="C54" s="13" t="inlineStr"/>
+      <c r="D54" s="13" t="inlineStr"/>
+      <c r="E54" s="13" t="inlineStr"/>
+      <c r="F54" s="13" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="10" t="n">
+      <c r="A55" s="11" t="n">
         <v>1969</v>
       </c>
-      <c r="B55" s="11" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>New York, NY; Missing</t>
         </is>
       </c>
-      <c r="C55" s="12" t="inlineStr"/>
-      <c r="D55" s="12" t="inlineStr"/>
-      <c r="E55" s="12" t="inlineStr"/>
-      <c r="F55" s="12" t="inlineStr"/>
+      <c r="C55" s="13" t="inlineStr"/>
+      <c r="D55" s="13" t="inlineStr"/>
+      <c r="E55" s="13" t="inlineStr"/>
+      <c r="F55" s="13" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="10" t="n">
+      <c r="A56" s="11" t="n">
         <v>1970</v>
       </c>
-      <c r="B56" s="11" t="inlineStr">
+      <c r="B56" s="12" t="inlineStr">
         <is>
           <t>New Orleans, LA; Missing</t>
         </is>
       </c>
-      <c r="C56" s="12" t="inlineStr"/>
-      <c r="D56" s="12" t="inlineStr"/>
-      <c r="E56" s="12" t="inlineStr"/>
-      <c r="F56" s="12" t="inlineStr"/>
+      <c r="C56" s="13" t="inlineStr"/>
+      <c r="D56" s="13" t="inlineStr"/>
+      <c r="E56" s="13" t="inlineStr"/>
+      <c r="F56" s="13" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="10" t="n">
+      <c r="A57" s="11" t="n">
         <v>1971</v>
       </c>
-      <c r="B57" s="11" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>Los Angeles, CA; Missing</t>
         </is>
       </c>
-      <c r="C57" s="12" t="inlineStr"/>
-      <c r="D57" s="12" t="inlineStr"/>
-      <c r="E57" s="12" t="inlineStr"/>
-      <c r="F57" s="12" t="inlineStr"/>
+      <c r="C57" s="13" t="inlineStr"/>
+      <c r="D57" s="13" t="inlineStr"/>
+      <c r="E57" s="13" t="inlineStr"/>
+      <c r="F57" s="13" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="10" t="n">
+      <c r="A58" s="11" t="n">
         <v>1972</v>
       </c>
-      <c r="B58" s="11" t="inlineStr">
+      <c r="B58" s="12" t="inlineStr">
         <is>
           <t>Boston, MA; Missing</t>
         </is>
       </c>
-      <c r="C58" s="12" t="inlineStr"/>
-      <c r="D58" s="12" t="inlineStr"/>
-      <c r="E58" s="12" t="inlineStr"/>
-      <c r="F58" s="12" t="inlineStr"/>
+      <c r="C58" s="13" t="inlineStr"/>
+      <c r="D58" s="13" t="inlineStr"/>
+      <c r="E58" s="13" t="inlineStr"/>
+      <c r="F58" s="13" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="10" t="n">
+      <c r="A59" s="11" t="n">
         <v>1973</v>
       </c>
-      <c r="B59" s="11" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>San Jose, Costa Rica; Missing</t>
         </is>
       </c>
-      <c r="C59" s="12" t="inlineStr"/>
-      <c r="D59" s="12" t="inlineStr"/>
-      <c r="E59" s="12" t="inlineStr"/>
-      <c r="F59" s="12" t="inlineStr"/>
+      <c r="C59" s="13" t="inlineStr"/>
+      <c r="D59" s="13" t="inlineStr"/>
+      <c r="E59" s="13" t="inlineStr"/>
+      <c r="F59" s="13" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="10" t="n">
+      <c r="A60" s="11" t="n">
         <v>1974</v>
       </c>
-      <c r="B60" s="11" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
         <is>
           <t>Ottawa, ON; Missing</t>
         </is>
       </c>
-      <c r="C60" s="12" t="inlineStr"/>
-      <c r="D60" s="12" t="inlineStr"/>
-      <c r="E60" s="12" t="inlineStr"/>
-      <c r="F60" s="12" t="inlineStr"/>
+      <c r="C60" s="13" t="inlineStr"/>
+      <c r="D60" s="13" t="inlineStr"/>
+      <c r="E60" s="13" t="inlineStr"/>
+      <c r="F60" s="13" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="10" t="n">
+      <c r="A61" s="11" t="n">
         <v>1975</v>
       </c>
-      <c r="B61" s="11" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>Williamsburg, VA; Missing</t>
         </is>
       </c>
-      <c r="C61" s="12" t="inlineStr"/>
-      <c r="D61" s="12" t="inlineStr"/>
-      <c r="E61" s="12" t="inlineStr"/>
-      <c r="F61" s="12" t="inlineStr"/>
+      <c r="C61" s="13" t="inlineStr"/>
+      <c r="D61" s="13" t="inlineStr"/>
+      <c r="E61" s="13" t="inlineStr"/>
+      <c r="F61" s="13" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="10" t="n">
+      <c r="A62" s="11" t="n">
         <v>1976</v>
       </c>
-      <c r="B62" s="11" t="inlineStr">
+      <c r="B62" s="12" t="inlineStr">
         <is>
           <t>Fairbanks, AK; Missing</t>
         </is>
       </c>
-      <c r="C62" s="12" t="inlineStr"/>
-      <c r="D62" s="12" t="inlineStr"/>
-      <c r="E62" s="12" t="inlineStr"/>
-      <c r="F62" s="12" t="inlineStr"/>
+      <c r="C62" s="13" t="inlineStr"/>
+      <c r="D62" s="13" t="inlineStr"/>
+      <c r="E62" s="13" t="inlineStr"/>
+      <c r="F62" s="13" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="10" t="n">
+      <c r="A63" s="11" t="n">
         <v>1977</v>
       </c>
-      <c r="B63" s="11" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>Gainesville, FL; Missing</t>
         </is>
       </c>
-      <c r="C63" s="12" t="inlineStr"/>
-      <c r="D63" s="12" t="inlineStr"/>
-      <c r="E63" s="12" t="inlineStr"/>
-      <c r="F63" s="12" t="inlineStr"/>
+      <c r="C63" s="13" t="inlineStr"/>
+      <c r="D63" s="13" t="inlineStr"/>
+      <c r="E63" s="13" t="inlineStr"/>
+      <c r="F63" s="13" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="10" t="n">
+      <c r="A64" s="11" t="n">
         <v>1978</v>
       </c>
-      <c r="B64" s="11" t="inlineStr">
+      <c r="B64" s="12" t="inlineStr">
         <is>
           <t>Tempe, AZ; Missing</t>
         </is>
       </c>
-      <c r="C64" s="12" t="inlineStr"/>
-      <c r="D64" s="12" t="inlineStr"/>
-      <c r="E64" s="12" t="inlineStr"/>
-      <c r="F64" s="12" t="inlineStr"/>
+      <c r="C64" s="13" t="inlineStr"/>
+      <c r="D64" s="13" t="inlineStr"/>
+      <c r="E64" s="13" t="inlineStr"/>
+      <c r="F64" s="13" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="10" t="n">
+      <c r="A65" s="11" t="n">
         <v>1979</v>
       </c>
-      <c r="B65" s="11" t="inlineStr">
+      <c r="B65" s="12" t="inlineStr">
         <is>
           <t>Orono, ME; Missing</t>
         </is>
       </c>
-      <c r="C65" s="12" t="inlineStr"/>
-      <c r="D65" s="12" t="inlineStr"/>
-      <c r="E65" s="12" t="inlineStr"/>
-      <c r="F65" s="12" t="inlineStr"/>
+      <c r="C65" s="13" t="inlineStr"/>
+      <c r="D65" s="13" t="inlineStr"/>
+      <c r="E65" s="13" t="inlineStr"/>
+      <c r="F65" s="13" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="10" t="n">
+      <c r="A66" s="11" t="n">
         <v>1980</v>
       </c>
-      <c r="B66" s="11" t="inlineStr">
+      <c r="B66" s="12" t="inlineStr">
         <is>
           <t>Fort Worth, TX; Missing</t>
         </is>
       </c>
-      <c r="C66" s="12" t="inlineStr"/>
-      <c r="D66" s="12" t="inlineStr"/>
-      <c r="E66" s="12" t="inlineStr"/>
-      <c r="F66" s="12" t="inlineStr"/>
+      <c r="C66" s="13" t="inlineStr"/>
+      <c r="D66" s="13" t="inlineStr"/>
+      <c r="E66" s="13" t="inlineStr"/>
+      <c r="F66" s="13" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="10" t="n">
+      <c r="A67" s="11" t="n">
         <v>1981</v>
       </c>
-      <c r="B67" s="11" t="inlineStr">
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>Corvallis, OR; Missing</t>
         </is>
       </c>
-      <c r="C67" s="12" t="inlineStr"/>
-      <c r="D67" s="12" t="inlineStr"/>
-      <c r="E67" s="12" t="inlineStr"/>
-      <c r="F67" s="12" t="inlineStr"/>
+      <c r="C67" s="13" t="inlineStr"/>
+      <c r="D67" s="13" t="inlineStr"/>
+      <c r="E67" s="13" t="inlineStr"/>
+      <c r="F67" s="13" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="10" t="n">
+      <c r="A68" s="11" t="n">
         <v>1982</v>
       </c>
-      <c r="B68" s="11" t="inlineStr">
+      <c r="B68" s="12" t="inlineStr">
         <is>
           <t>DeKalb, IL; Missing</t>
         </is>
       </c>
-      <c r="C68" s="12" t="inlineStr"/>
-      <c r="D68" s="12" t="inlineStr"/>
-      <c r="E68" s="12" t="inlineStr"/>
-      <c r="F68" s="12" t="inlineStr"/>
+      <c r="C68" s="13" t="inlineStr"/>
+      <c r="D68" s="13" t="inlineStr"/>
+      <c r="E68" s="13" t="inlineStr"/>
+      <c r="F68" s="13" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="10" t="n">
+      <c r="A69" s="11" t="n">
         <v>1983</v>
       </c>
-      <c r="B69" s="11" t="inlineStr">
+      <c r="B69" s="12" t="inlineStr">
         <is>
           <t>Tallahasee, FL; Missing</t>
         </is>
       </c>
-      <c r="C69" s="11" t="inlineStr">
+      <c r="C69" s="12" t="inlineStr">
         <is>
           <t>Tallahasee, FL; Missing</t>
         </is>
       </c>
-      <c r="D69" s="12" t="inlineStr"/>
-      <c r="E69" s="12" t="inlineStr"/>
-      <c r="F69" s="12" t="inlineStr"/>
+      <c r="D69" s="13" t="inlineStr"/>
+      <c r="E69" s="13" t="inlineStr"/>
+      <c r="F69" s="13" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="10" t="n">
+      <c r="A70" s="11" t="n">
         <v>1984</v>
       </c>
-      <c r="B70" s="11" t="inlineStr">
+      <c r="B70" s="12" t="inlineStr">
         <is>
           <t>Norman, OK; Missing</t>
         </is>
       </c>
-      <c r="C70" s="11" t="inlineStr">
+      <c r="C70" s="12" t="inlineStr">
         <is>
           <t>Norman, OK; Missing</t>
         </is>
       </c>
-      <c r="D70" s="12" t="inlineStr"/>
-      <c r="E70" s="12" t="inlineStr"/>
-      <c r="F70" s="12" t="inlineStr"/>
+      <c r="D70" s="13" t="inlineStr"/>
+      <c r="E70" s="13" t="inlineStr"/>
+      <c r="F70" s="13" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="10" t="n">
+      <c r="A71" s="11" t="n">
         <v>1985</v>
       </c>
-      <c r="B71" s="11" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
         <is>
           <t>Knoxville, TN; Missing</t>
         </is>
       </c>
-      <c r="C71" s="11" t="inlineStr">
+      <c r="C71" s="12" t="inlineStr">
         <is>
           <t>Knoxville, TN; Missing</t>
         </is>
       </c>
-      <c r="D71" s="12" t="inlineStr"/>
-      <c r="E71" s="12" t="inlineStr"/>
-      <c r="F71" s="12" t="inlineStr"/>
+      <c r="D71" s="13" t="inlineStr"/>
+      <c r="E71" s="13" t="inlineStr"/>
+      <c r="F71" s="13" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="10" t="n">
+      <c r="A72" s="11" t="n">
         <v>1986</v>
       </c>
-      <c r="B72" s="11" t="inlineStr">
+      <c r="B72" s="12" t="inlineStr">
         <is>
           <t>Victoria, BC; Missing</t>
         </is>
       </c>
-      <c r="C72" s="11" t="inlineStr">
+      <c r="C72" s="12" t="inlineStr">
         <is>
           <t>Victoria, BC; Missing</t>
         </is>
       </c>
-      <c r="D72" s="12" t="inlineStr"/>
-      <c r="E72" s="12" t="inlineStr"/>
-      <c r="F72" s="12" t="inlineStr"/>
+      <c r="D72" s="13" t="inlineStr"/>
+      <c r="E72" s="13" t="inlineStr"/>
+      <c r="F72" s="13" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="10" t="n">
+      <c r="A73" s="11" t="n">
         <v>1987</v>
       </c>
-      <c r="B73" s="11" t="inlineStr">
+      <c r="B73" s="12" t="inlineStr">
         <is>
           <t>Albany, NY; Missing</t>
         </is>
       </c>
-      <c r="C73" s="11" t="inlineStr">
+      <c r="C73" s="12" t="inlineStr">
         <is>
           <t>Albany, NY; Missing</t>
         </is>
       </c>
-      <c r="D73" s="12" t="inlineStr"/>
-      <c r="E73" s="12" t="inlineStr"/>
-      <c r="F73" s="12" t="inlineStr"/>
+      <c r="D73" s="13" t="inlineStr"/>
+      <c r="E73" s="13" t="inlineStr"/>
+      <c r="F73" s="13" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="10" t="n">
+      <c r="A74" s="11" t="n">
         <v>1988</v>
       </c>
-      <c r="B74" s="11" t="inlineStr">
+      <c r="B74" s="12" t="inlineStr">
         <is>
           <t>Ann Arbor, MI; Missing</t>
         </is>
       </c>
-      <c r="C74" s="11" t="inlineStr">
+      <c r="C74" s="12" t="inlineStr">
         <is>
           <t>Ann Arbor, MI; Missing</t>
         </is>
       </c>
-      <c r="D74" s="12" t="inlineStr"/>
-      <c r="E74" s="12" t="inlineStr"/>
-      <c r="F74" s="12" t="inlineStr"/>
+      <c r="D74" s="13" t="inlineStr"/>
+      <c r="E74" s="13" t="inlineStr"/>
+      <c r="F74" s="13" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="10" t="n">
+      <c r="A75" s="11" t="n">
         <v>1989</v>
       </c>
-      <c r="B75" s="11" t="inlineStr">
+      <c r="B75" s="12" t="inlineStr">
         <is>
           <t>San Francisco, CA; Missing</t>
         </is>
       </c>
-      <c r="C75" s="11" t="inlineStr">
+      <c r="C75" s="12" t="inlineStr">
         <is>
           <t>San Francisco, CA; Missing</t>
         </is>
       </c>
-      <c r="D75" s="12" t="inlineStr"/>
-      <c r="E75" s="12" t="inlineStr"/>
-      <c r="F75" s="12" t="inlineStr"/>
+      <c r="D75" s="13" t="inlineStr"/>
+      <c r="E75" s="13" t="inlineStr"/>
+      <c r="F75" s="13" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="10" t="n">
+      <c r="A76" s="11" t="n">
         <v>1990</v>
       </c>
-      <c r="B76" s="11" t="inlineStr">
+      <c r="B76" s="12" t="inlineStr">
         <is>
           <t>Charleston, SC; Missing</t>
         </is>
       </c>
-      <c r="C76" s="11" t="inlineStr">
+      <c r="C76" s="12" t="inlineStr">
         <is>
           <t>Charleston, SC; Missing</t>
         </is>
       </c>
-      <c r="D76" s="12" t="inlineStr"/>
-      <c r="E76" s="12" t="inlineStr"/>
-      <c r="F76" s="12" t="inlineStr"/>
+      <c r="D76" s="13" t="inlineStr"/>
+      <c r="E76" s="13" t="inlineStr"/>
+      <c r="F76" s="13" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="10" t="n">
+      <c r="A77" s="11" t="n">
         <v>1991</v>
       </c>
-      <c r="B77" s="11" t="inlineStr">
+      <c r="B77" s="12" t="inlineStr">
         <is>
           <t>New York, NY; Missing</t>
         </is>
       </c>
-      <c r="C77" s="11" t="inlineStr">
+      <c r="C77" s="12" t="inlineStr">
         <is>
           <t>New York, NY; Missing</t>
         </is>
       </c>
-      <c r="D77" s="12" t="inlineStr"/>
-      <c r="E77" s="12" t="inlineStr"/>
-      <c r="F77" s="12" t="inlineStr"/>
+      <c r="D77" s="13" t="inlineStr"/>
+      <c r="E77" s="13" t="inlineStr"/>
+      <c r="F77" s="13" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="10" t="n">
+      <c r="A78" s="11" t="n">
         <v>1992</v>
       </c>
-      <c r="B78" s="13" t="inlineStr">
-        <is>
-          <t>Champaign-Urbana, IL; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C78" s="13" t="inlineStr">
-        <is>
-          <t>Champaign-Urbana, IL; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D78" s="12" t="inlineStr"/>
-      <c r="E78" s="12" t="inlineStr"/>
-      <c r="F78" s="12" t="inlineStr"/>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>Champaign-Urbana, IL; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>Champaign-Urbana, IL; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D78" s="13" t="inlineStr"/>
+      <c r="E78" s="13" t="inlineStr"/>
+      <c r="F78" s="13" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="10" t="n">
+      <c r="A79" s="11" t="n">
         <v>1993</v>
       </c>
-      <c r="B79" s="13" t="inlineStr">
-        <is>
-          <t>Austin, TX; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C79" s="13" t="inlineStr">
-        <is>
-          <t>Austin, TX; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D79" s="12" t="inlineStr"/>
-      <c r="E79" s="12" t="inlineStr"/>
-      <c r="F79" s="12" t="inlineStr"/>
+      <c r="B79" s="14" t="inlineStr">
+        <is>
+          <t>Austin, TX; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C79" s="14" t="inlineStr">
+        <is>
+          <t>Austin, TX; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D79" s="13" t="inlineStr"/>
+      <c r="E79" s="13" t="inlineStr"/>
+      <c r="F79" s="13" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="10" t="n">
+      <c r="A80" s="11" t="n">
         <v>1994</v>
       </c>
-      <c r="B80" s="13" t="inlineStr">
-        <is>
-          <t>Los Angeles, CA; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C80" s="13" t="inlineStr">
-        <is>
-          <t>Los Angeles, CA; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D80" s="12" t="inlineStr"/>
-      <c r="E80" s="12" t="inlineStr"/>
-      <c r="F80" s="12" t="inlineStr"/>
+      <c r="B80" s="14" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C80" s="14" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D80" s="13" t="inlineStr"/>
+      <c r="E80" s="13" t="inlineStr"/>
+      <c r="F80" s="13" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="10" t="n">
+      <c r="A81" s="11" t="n">
         <v>1995</v>
       </c>
-      <c r="B81" s="13" t="inlineStr">
-        <is>
-          <t>Edmonton, AB; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C81" s="13" t="inlineStr">
-        <is>
-          <t>Edmonton, AB; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D81" s="12" t="inlineStr"/>
-      <c r="E81" s="12" t="inlineStr"/>
-      <c r="F81" s="12" t="inlineStr"/>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>Edmonton, AB; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>Edmonton, AB; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D81" s="13" t="inlineStr"/>
+      <c r="E81" s="13" t="inlineStr"/>
+      <c r="F81" s="13" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="10" t="n">
+      <c r="A82" s="11" t="n">
         <v>1996</v>
       </c>
-      <c r="B82" s="13" t="inlineStr">
-        <is>
-          <t>New Orleans, LA; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C82" s="13" t="inlineStr">
-        <is>
-          <t>New Orleans, LA; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D82" s="12" t="inlineStr"/>
-      <c r="E82" s="12" t="inlineStr"/>
-      <c r="F82" s="12" t="inlineStr"/>
+      <c r="B82" s="14" t="inlineStr">
+        <is>
+          <t>New Orleans, LA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C82" s="14" t="inlineStr">
+        <is>
+          <t>New Orleans, LA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D82" s="13" t="inlineStr"/>
+      <c r="E82" s="13" t="inlineStr"/>
+      <c r="F82" s="13" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="10" t="n">
+      <c r="A83" s="11" t="n">
         <v>1997</v>
       </c>
-      <c r="B83" s="14" t="inlineStr">
-        <is>
-          <t>Seattle, WA; OCR</t>
-        </is>
-      </c>
-      <c r="C83" s="14" t="inlineStr">
-        <is>
-          <t>Seattle, WA (58); OCR</t>
-        </is>
-      </c>
-      <c r="D83" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E83" s="12" t="inlineStr"/>
-      <c r="F83" s="12" t="inlineStr"/>
+      <c r="B83" s="15" t="inlineStr">
+        <is>
+          <t>Seattle, WA; OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
+        </is>
+      </c>
+      <c r="C83" s="15" t="inlineStr">
+        <is>
+          <t>Seattle, WA (58); OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
+        </is>
+      </c>
+      <c r="D83" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E83" s="13" t="inlineStr"/>
+      <c r="F83" s="13" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="10" t="n">
+      <c r="A84" s="11" t="n">
         <v>1998</v>
       </c>
-      <c r="B84" s="14" t="inlineStr">
-        <is>
-          <t>Guelph, ON; OCR</t>
-        </is>
-      </c>
-      <c r="C84" s="14" t="inlineStr">
-        <is>
-          <t>Guelph, ON (15); OCR</t>
-        </is>
-      </c>
-      <c r="D84" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E84" s="12" t="inlineStr"/>
-      <c r="F84" s="12" t="inlineStr"/>
+      <c r="B84" s="15" t="inlineStr">
+        <is>
+          <t>Guelph, ON; OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
+        </is>
+      </c>
+      <c r="C84" s="15" t="inlineStr">
+        <is>
+          <t>Guelph, ON (15); OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
+        </is>
+      </c>
+      <c r="D84" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E84" s="13" t="inlineStr"/>
+      <c r="F84" s="13" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="10" t="n">
+      <c r="A85" s="11" t="n">
         <v>1999</v>
       </c>
-      <c r="B85" s="14" t="inlineStr">
-        <is>
-          <t>University Park, PA; OCR</t>
-        </is>
-      </c>
-      <c r="C85" s="14" t="inlineStr">
-        <is>
-          <t>University Park, PA (57); OCR</t>
-        </is>
-      </c>
-      <c r="D85" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E85" s="12" t="inlineStr"/>
-      <c r="F85" s="12" t="inlineStr"/>
+      <c r="B85" s="15" t="inlineStr">
+        <is>
+          <t>University Park, PA; OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
+        </is>
+      </c>
+      <c r="C85" s="15" t="inlineStr">
+        <is>
+          <t>University Park, PA (57); OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
+        </is>
+      </c>
+      <c r="D85" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E85" s="13" t="inlineStr"/>
+      <c r="F85" s="13" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="10" t="n">
+      <c r="A86" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="B86" s="14" t="inlineStr">
-        <is>
-          <t>La Paz, Mexico; OCR</t>
-        </is>
-      </c>
-      <c r="C86" s="14" t="inlineStr">
-        <is>
-          <t>La Paz, Mexico (59); OCR</t>
-        </is>
-      </c>
-      <c r="D86" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E86" s="12" t="inlineStr"/>
-      <c r="F86" s="12" t="inlineStr"/>
+      <c r="B86" s="15" t="inlineStr">
+        <is>
+          <t>La Paz, Mexico; OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
+        </is>
+      </c>
+      <c r="C86" s="15" t="inlineStr">
+        <is>
+          <t>La Paz, Mexico (59); OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
+        </is>
+      </c>
+      <c r="D86" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E86" s="13" t="inlineStr"/>
+      <c r="F86" s="13" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="10" t="n">
+      <c r="A87" s="11" t="n">
         <v>2001</v>
       </c>
-      <c r="B87" s="14" t="inlineStr">
-        <is>
-          <t>University Park, PA; OCR</t>
-        </is>
-      </c>
-      <c r="C87" s="14" t="inlineStr">
-        <is>
-          <t>University Park, PA (67); OCR</t>
-        </is>
-      </c>
-      <c r="D87" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E87" s="12" t="inlineStr"/>
-      <c r="F87" s="12" t="inlineStr"/>
+      <c r="B87" s="15" t="inlineStr">
+        <is>
+          <t>University Park, PA; OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
+        </is>
+      </c>
+      <c r="C87" s="15" t="inlineStr">
+        <is>
+          <t>University Park, PA (67); OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
+        </is>
+      </c>
+      <c r="D87" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E87" s="13" t="inlineStr"/>
+      <c r="F87" s="13" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="10" t="n">
+      <c r="A88" s="11" t="n">
         <v>2002</v>
       </c>
-      <c r="B88" s="13" t="inlineStr">
-        <is>
-          <t>Kansas City, MO; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C88" s="13" t="inlineStr">
-        <is>
-          <t>Kansas City, MO; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D88" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E88" s="12" t="inlineStr"/>
-      <c r="F88" s="12" t="inlineStr"/>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>Kansas City, MO; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>Kansas City, MO; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E88" s="13" t="inlineStr"/>
+      <c r="F88" s="13" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="10" t="n">
+      <c r="A89" s="11" t="n">
         <v>2003</v>
       </c>
-      <c r="B89" s="13" t="inlineStr">
-        <is>
-          <t>Manaus, Brazil; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C89" s="13" t="inlineStr">
-        <is>
-          <t>Manaus, Brazil; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D89" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E89" s="12" t="inlineStr"/>
-      <c r="F89" s="12" t="inlineStr"/>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>Manaus, Brazil; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>Manaus, Brazil; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D89" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E89" s="13" t="inlineStr"/>
+      <c r="F89" s="13" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="10" t="n">
+      <c r="A90" s="11" t="n">
         <v>2004</v>
       </c>
-      <c r="B90" s="13" t="inlineStr">
-        <is>
-          <t>Norman, OK; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C90" s="13" t="inlineStr">
-        <is>
-          <t>Norman, OK; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D90" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E90" s="12" t="inlineStr"/>
-      <c r="F90" s="12" t="inlineStr"/>
+      <c r="B90" s="14" t="inlineStr">
+        <is>
+          <t>Norman, OK; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>Norman, OK; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E90" s="13" t="inlineStr"/>
+      <c r="F90" s="13" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="10" t="n">
+      <c r="A91" s="11" t="n">
         <v>2005</v>
       </c>
-      <c r="B91" s="15" t="inlineStr">
+      <c r="B91" s="16" t="inlineStr">
         <is>
           <t>Tampa, FL; Ingested</t>
         </is>
       </c>
-      <c r="C91" s="15" t="inlineStr">
+      <c r="C91" s="16" t="inlineStr">
         <is>
           <t>Tampa, FL (80); Ingested</t>
         </is>
       </c>
-      <c r="D91" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E91" s="12" t="inlineStr"/>
-      <c r="F91" s="12" t="inlineStr"/>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E91" s="13" t="inlineStr"/>
+      <c r="F91" s="13" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="10" t="n">
+      <c r="A92" s="11" t="n">
         <v>2006</v>
       </c>
-      <c r="B92" s="13" t="inlineStr">
-        <is>
-          <t>New Orleans, LA; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C92" s="13" t="inlineStr">
-        <is>
-          <t>New Orleans, LA; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D92" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E92" s="12" t="inlineStr"/>
-      <c r="F92" s="12" t="inlineStr"/>
+      <c r="B92" s="14" t="inlineStr">
+        <is>
+          <t>New Orleans, LA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>New Orleans, LA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D92" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E92" s="13" t="inlineStr"/>
+      <c r="F92" s="13" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="10" t="n">
+      <c r="A93" s="11" t="n">
         <v>2007</v>
       </c>
-      <c r="B93" s="15" t="inlineStr">
+      <c r="B93" s="16" t="inlineStr">
         <is>
           <t>St. Louis, MO; Ingested</t>
         </is>
       </c>
-      <c r="C93" s="15" t="inlineStr">
+      <c r="C93" s="16" t="inlineStr">
         <is>
           <t>St. Louis, MO (155); Ingested</t>
         </is>
       </c>
-      <c r="D93" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E93" s="12" t="inlineStr"/>
-      <c r="F93" s="12" t="inlineStr"/>
+      <c r="D93" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E93" s="13" t="inlineStr"/>
+      <c r="F93" s="13" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="10" t="n">
+      <c r="A94" s="11" t="n">
         <v>2008</v>
       </c>
-      <c r="B94" s="16" t="inlineStr">
-        <is>
-          <t>Montreal, PQ; Schedule</t>
-        </is>
-      </c>
-      <c r="C94" s="16" t="inlineStr">
-        <is>
-          <t>Montreal, PQ (193); Schedule</t>
-        </is>
-      </c>
-      <c r="D94" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E94" s="12" t="inlineStr"/>
-      <c r="F94" s="12" t="inlineStr"/>
+      <c r="B94" s="17" t="inlineStr">
+        <is>
+          <t>Montreal, PQ; Schedule — programme ingested (no abstract bodies)</t>
+        </is>
+      </c>
+      <c r="C94" s="17" t="inlineStr">
+        <is>
+          <t>Montreal, PQ (193); Schedule — programme ingested (no abstract bodies)</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E94" s="13" t="inlineStr"/>
+      <c r="F94" s="13" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="10" t="n">
+      <c r="A95" s="11" t="n">
         <v>2009</v>
       </c>
-      <c r="B95" s="15" t="inlineStr">
+      <c r="B95" s="16" t="inlineStr">
         <is>
           <t>Portland, OR; Ingested</t>
         </is>
       </c>
-      <c r="C95" s="15" t="inlineStr">
+      <c r="C95" s="16" t="inlineStr">
         <is>
           <t>Portland, OR (149); Ingested</t>
         </is>
       </c>
-      <c r="D95" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy (Ali archive)</t>
-        </is>
-      </c>
-      <c r="E95" s="12" t="inlineStr"/>
-      <c r="F95" s="12" t="inlineStr"/>
+      <c r="D95" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+        </is>
+      </c>
+      <c r="E95" s="13" t="inlineStr"/>
+      <c r="F95" s="13" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="10" t="n">
+      <c r="A96" s="11" t="n">
         <v>2010</v>
       </c>
-      <c r="B96" s="13" t="inlineStr">
-        <is>
-          <t>Providence, RI; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C96" s="13" t="inlineStr">
-        <is>
-          <t>Providence, RI; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D96" s="13" t="inlineStr">
-        <is>
-          <t>Galway; Hardcopy</t>
-        </is>
-      </c>
-      <c r="E96" s="12" t="inlineStr"/>
-      <c r="F96" s="11" t="inlineStr">
-        <is>
-          <t>Cairns; Missing</t>
+      <c r="B96" s="14" t="inlineStr">
+        <is>
+          <t>Providence, RI; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C96" s="14" t="inlineStr">
+        <is>
+          <t>Providence, RI; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
+        <is>
+          <t>Galway; Hardcopy — Cat has hardcopy</t>
+        </is>
+      </c>
+      <c r="E96" s="13" t="inlineStr"/>
+      <c r="F96" s="12" t="inlineStr">
+        <is>
+          <t>Cairns; Missing — find source</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="10" t="n">
+      <c r="A97" s="11" t="n">
         <v>2011</v>
       </c>
-      <c r="B97" s="13" t="inlineStr">
-        <is>
-          <t>Minneapolis, MN; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C97" s="13" t="inlineStr">
-        <is>
-          <t>Minneapolis, MN; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D97" s="13" t="inlineStr">
-        <is>
-          <t>Berlin; Hardcopy</t>
-        </is>
-      </c>
-      <c r="E97" s="12" t="inlineStr"/>
-      <c r="F97" s="12" t="inlineStr"/>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>Minneapolis, MN; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C97" s="14" t="inlineStr">
+        <is>
+          <t>Minneapolis, MN; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D97" s="14" t="inlineStr">
+        <is>
+          <t>Berlin; Hardcopy — Cat has hardcopy</t>
+        </is>
+      </c>
+      <c r="E97" s="13" t="inlineStr"/>
+      <c r="F97" s="13" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="10" t="n">
+      <c r="A98" s="11" t="n">
         <v>2012</v>
       </c>
-      <c r="B98" s="15" t="inlineStr">
+      <c r="B98" s="16" t="inlineStr">
         <is>
           <t>Vancouver, BC; Ingested</t>
         </is>
       </c>
-      <c r="C98" s="15" t="inlineStr">
+      <c r="C98" s="16" t="inlineStr">
         <is>
           <t>Vancouver, BC (65); Ingested</t>
         </is>
       </c>
-      <c r="D98" s="13" t="inlineStr">
-        <is>
-          <t>Milan; Hardcopy</t>
-        </is>
-      </c>
-      <c r="E98" s="17" t="inlineStr">
-        <is>
-          <t>?; Pending (Brit)</t>
-        </is>
-      </c>
-      <c r="F98" s="12" t="inlineStr"/>
+      <c r="D98" s="14" t="inlineStr">
+        <is>
+          <t>Milan; Hardcopy — Cat has hardcopy</t>
+        </is>
+      </c>
+      <c r="E98" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Brit collating (council approval)</t>
+        </is>
+      </c>
+      <c r="F98" s="13" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="10" t="n">
+      <c r="A99" s="11" t="n">
         <v>2013</v>
       </c>
-      <c r="B99" s="13" t="inlineStr">
-        <is>
-          <t>Albuquerque, NM; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C99" s="13" t="inlineStr">
-        <is>
-          <t>Albuquerque, NM; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D99" s="18" t="inlineStr">
-        <is>
-          <t>Plymouth; Digital</t>
-        </is>
-      </c>
-      <c r="E99" s="12" t="inlineStr"/>
-      <c r="F99" s="12" t="inlineStr"/>
+      <c r="B99" s="14" t="inlineStr">
+        <is>
+          <t>Albuquerque, NM; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C99" s="14" t="inlineStr">
+        <is>
+          <t>Albuquerque, NM; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D99" s="19" t="inlineStr">
+        <is>
+          <t>Plymouth; Digital — abstract book held — ingest</t>
+        </is>
+      </c>
+      <c r="E99" s="13" t="inlineStr"/>
+      <c r="F99" s="13" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="10" t="n">
+      <c r="A100" s="11" t="n">
         <v>2014</v>
       </c>
-      <c r="B100" s="13" t="inlineStr">
-        <is>
-          <t>Chattanooga, TN; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C100" s="13" t="inlineStr">
-        <is>
-          <t>Chattanooga, TN; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D100" s="13" t="inlineStr">
-        <is>
-          <t>Leeuwarden; Hardcopy</t>
-        </is>
-      </c>
-      <c r="E100" s="17" t="inlineStr">
-        <is>
-          <t>?; Pending (Brit)</t>
-        </is>
-      </c>
-      <c r="F100" s="11" t="inlineStr">
-        <is>
-          <t>Durban; Missing</t>
+      <c r="B100" s="14" t="inlineStr">
+        <is>
+          <t>Chattanooga, TN; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C100" s="14" t="inlineStr">
+        <is>
+          <t>Chattanooga, TN; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D100" s="14" t="inlineStr">
+        <is>
+          <t>Leeuwarden; Hardcopy — Cat has hardcopy</t>
+        </is>
+      </c>
+      <c r="E100" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Brit collating (council approval)</t>
+        </is>
+      </c>
+      <c r="F100" s="12" t="inlineStr">
+        <is>
+          <t>Durban; Missing — find source</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="10" t="n">
+      <c r="A101" s="11" t="n">
         <v>2015</v>
       </c>
-      <c r="B101" s="15" t="inlineStr">
+      <c r="B101" s="16" t="inlineStr">
         <is>
           <t>Reno, NV; Ingested</t>
         </is>
       </c>
-      <c r="C101" s="15" t="inlineStr">
+      <c r="C101" s="16" t="inlineStr">
         <is>
           <t>Reno, NV (123); Ingested</t>
         </is>
       </c>
-      <c r="D101" s="18" t="inlineStr">
-        <is>
-          <t>Peniche; Digital</t>
-        </is>
-      </c>
-      <c r="E101" s="12" t="inlineStr"/>
-      <c r="F101" s="12" t="inlineStr"/>
+      <c r="D101" s="19" t="inlineStr">
+        <is>
+          <t>Peniche; Digital — abstract book held — ingest</t>
+        </is>
+      </c>
+      <c r="E101" s="13" t="inlineStr"/>
+      <c r="F101" s="13" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="10" t="n">
+      <c r="A102" s="11" t="n">
         <v>2016</v>
       </c>
-      <c r="B102" s="15" t="inlineStr">
+      <c r="B102" s="16" t="inlineStr">
         <is>
           <t>New Orleans, LA; Ingested</t>
         </is>
       </c>
-      <c r="C102" s="15" t="inlineStr">
+      <c r="C102" s="16" t="inlineStr">
         <is>
           <t>New Orleans, LA (240); Ingested</t>
         </is>
       </c>
-      <c r="D102" s="13" t="inlineStr">
-        <is>
-          <t>Bristol; Hardcopy</t>
-        </is>
-      </c>
-      <c r="E102" s="17" t="inlineStr">
-        <is>
-          <t>?; Pending (Brit)</t>
-        </is>
-      </c>
-      <c r="F102" s="12" t="inlineStr"/>
+      <c r="D102" s="14" t="inlineStr">
+        <is>
+          <t>Bristol; Hardcopy — Cat (Shark Trust) hosted — ask for print PDF</t>
+        </is>
+      </c>
+      <c r="E102" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Brit collating (council approval)</t>
+        </is>
+      </c>
+      <c r="F102" s="13" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="10" t="n">
+      <c r="A103" s="11" t="n">
         <v>2017</v>
       </c>
-      <c r="B103" s="18" t="inlineStr">
-        <is>
-          <t>Austin, TX; Digital</t>
-        </is>
-      </c>
-      <c r="C103" s="18" t="inlineStr">
-        <is>
-          <t>Austin, TX; Digital</t>
-        </is>
-      </c>
-      <c r="D103" s="18" t="inlineStr">
-        <is>
-          <t>Amsterdam; Digital</t>
-        </is>
-      </c>
-      <c r="E103" s="12" t="inlineStr"/>
-      <c r="F103" s="12" t="inlineStr"/>
+      <c r="B103" s="20" t="inlineStr">
+        <is>
+          <t>Austin, TX; Programme — grid programme only — abstract book needed (Carylanne)</t>
+        </is>
+      </c>
+      <c r="C103" s="20" t="inlineStr">
+        <is>
+          <t>Austin, TX; Programme — grid programme only — abstract book needed (Carylanne)</t>
+        </is>
+      </c>
+      <c r="D103" s="20" t="inlineStr">
+        <is>
+          <t>Amsterdam; Programme — only programme held — abstract book needed</t>
+        </is>
+      </c>
+      <c r="E103" s="13" t="inlineStr"/>
+      <c r="F103" s="13" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="10" t="n">
+      <c r="A104" s="11" t="n">
         <v>2018</v>
       </c>
-      <c r="B104" s="13" t="inlineStr">
-        <is>
-          <t>Rochester, NY; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C104" s="13" t="inlineStr">
-        <is>
-          <t>Rochester, NY; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D104" s="18" t="inlineStr">
-        <is>
-          <t>Peniche; Digital</t>
-        </is>
-      </c>
-      <c r="E104" s="17" t="inlineStr">
-        <is>
-          <t>?; Pending (Brit)</t>
-        </is>
-      </c>
-      <c r="F104" s="15" t="inlineStr">
+      <c r="B104" s="14" t="inlineStr">
+        <is>
+          <t>Rochester, NY; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C104" s="14" t="inlineStr">
+        <is>
+          <t>Rochester, NY; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D104" s="12" t="inlineStr">
+        <is>
+          <t>Peniche; Missing — Cat: no hardcopy, likely online-only — find</t>
+        </is>
+      </c>
+      <c r="E104" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Brit collating (council approval)</t>
+        </is>
+      </c>
+      <c r="F104" s="16" t="inlineStr">
         <is>
           <t>Joao Pessoa; Ingested</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="10" t="n">
+      <c r="A105" s="11" t="n">
         <v>2019</v>
       </c>
-      <c r="B105" s="18" t="inlineStr">
-        <is>
-          <t>Snowbird, UT; Digital</t>
-        </is>
-      </c>
-      <c r="C105" s="18" t="inlineStr">
-        <is>
-          <t>Snowbird, UT; Digital</t>
-        </is>
-      </c>
-      <c r="D105" s="13" t="inlineStr">
-        <is>
-          <t>Rende; Hardcopy</t>
-        </is>
-      </c>
-      <c r="E105" s="12" t="inlineStr"/>
-      <c r="F105" s="12" t="inlineStr"/>
+      <c r="B105" s="20" t="inlineStr">
+        <is>
+          <t>Snowbird, UT; Programme — grid programme only — abstract book needed (Carylanne)</t>
+        </is>
+      </c>
+      <c r="C105" s="20" t="inlineStr">
+        <is>
+          <t>Snowbird, UT; Programme — grid programme only — abstract book needed (Carylanne)</t>
+        </is>
+      </c>
+      <c r="D105" s="14" t="inlineStr">
+        <is>
+          <t>Rende; Hardcopy — Cat has hardcopy</t>
+        </is>
+      </c>
+      <c r="E105" s="13" t="inlineStr"/>
+      <c r="F105" s="13" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" s="10" t="n">
+      <c r="A106" s="11" t="n">
         <v>2020</v>
       </c>
-      <c r="B106" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy</t>
-        </is>
-      </c>
-      <c r="C106" s="13" t="inlineStr">
-        <is>
-          <t>?; Hardcopy</t>
-        </is>
-      </c>
-      <c r="D106" s="18" t="inlineStr">
-        <is>
-          <t>online (covid); Digital</t>
-        </is>
-      </c>
-      <c r="E106" s="17" t="inlineStr">
-        <is>
-          <t>?; Pending (Brit)</t>
-        </is>
-      </c>
-      <c r="F106" s="12" t="inlineStr"/>
+      <c r="B106" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="C106" s="14" t="inlineStr">
+        <is>
+          <t>?; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+        </is>
+      </c>
+      <c r="D106" s="12" t="inlineStr">
+        <is>
+          <t>online (covid); Missing — covid/online — find</t>
+        </is>
+      </c>
+      <c r="E106" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Brit collating (council approval)</t>
+        </is>
+      </c>
+      <c r="F106" s="13" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" s="10" t="n">
+      <c r="A107" s="11" t="n">
         <v>2021</v>
       </c>
-      <c r="B107" s="16" t="inlineStr">
-        <is>
-          <t>Phoenix, AZ; Schedule</t>
-        </is>
-      </c>
-      <c r="C107" s="16" t="inlineStr">
-        <is>
-          <t>Phoenix, AZ (46); Schedule</t>
-        </is>
-      </c>
-      <c r="D107" s="18" t="inlineStr">
-        <is>
-          <t>Leiden; Digital</t>
-        </is>
-      </c>
-      <c r="E107" s="12" t="inlineStr"/>
-      <c r="F107" s="12" t="inlineStr"/>
+      <c r="B107" s="17" t="inlineStr">
+        <is>
+          <t>Phoenix, AZ; Schedule — programme ingested (no abstract bodies)</t>
+        </is>
+      </c>
+      <c r="C107" s="17" t="inlineStr">
+        <is>
+          <t>Phoenix, AZ (46); Schedule — programme ingested (no abstract bodies)</t>
+        </is>
+      </c>
+      <c r="D107" s="20" t="inlineStr">
+        <is>
+          <t>Leiden; Programme — only programme held — abstract book needed</t>
+        </is>
+      </c>
+      <c r="E107" s="13" t="inlineStr"/>
+      <c r="F107" s="13" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" s="10" t="n">
+      <c r="A108" s="11" t="n">
         <v>2022</v>
       </c>
-      <c r="B108" s="16" t="inlineStr">
-        <is>
-          <t>Spokane, WA; Schedule</t>
-        </is>
-      </c>
-      <c r="C108" s="16" t="inlineStr">
-        <is>
-          <t>Spokane, WA (69); Schedule</t>
-        </is>
-      </c>
-      <c r="D108" s="18" t="inlineStr">
-        <is>
-          <t>Valencia (SI); Digital</t>
-        </is>
-      </c>
-      <c r="E108" s="17" t="inlineStr">
-        <is>
-          <t>?; Pending (Brit)</t>
-        </is>
-      </c>
-      <c r="F108" s="15" t="inlineStr">
-        <is>
-          <t>Valencia; Ingested</t>
+      <c r="B108" s="17" t="inlineStr">
+        <is>
+          <t>Spokane, WA; Schedule — programme ingested (no abstract bodies)</t>
+        </is>
+      </c>
+      <c r="C108" s="17" t="inlineStr">
+        <is>
+          <t>Spokane, WA (69); Schedule — programme ingested (no abstract bodies)</t>
+        </is>
+      </c>
+      <c r="D108" s="17" t="inlineStr">
+        <is>
+          <t>Valencia (=SI2022); Schedule — covered via SI2022 (schedule)</t>
+        </is>
+      </c>
+      <c r="E108" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Brit collating (council approval)</t>
+        </is>
+      </c>
+      <c r="F108" s="17" t="inlineStr">
+        <is>
+          <t>Valencia; Schedule — programme ingested (no bodies)</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="10" t="n">
+      <c r="A109" s="11" t="n">
         <v>2023</v>
       </c>
-      <c r="B109" s="16" t="inlineStr">
-        <is>
-          <t>Norfolk, VA; Schedule</t>
-        </is>
-      </c>
-      <c r="C109" s="16" t="inlineStr">
-        <is>
-          <t>Norfolk, VA (87); Schedule</t>
-        </is>
-      </c>
-      <c r="D109" s="18" t="inlineStr">
-        <is>
-          <t>Brighton; Digital</t>
-        </is>
-      </c>
-      <c r="E109" s="12" t="inlineStr"/>
-      <c r="F109" s="12" t="inlineStr"/>
+      <c r="B109" s="17" t="inlineStr">
+        <is>
+          <t>Norfolk, VA; Schedule — programme ingested (no abstract bodies)</t>
+        </is>
+      </c>
+      <c r="C109" s="17" t="inlineStr">
+        <is>
+          <t>Norfolk, VA (87); Schedule — programme ingested (no abstract bodies)</t>
+        </is>
+      </c>
+      <c r="D109" s="20" t="inlineStr">
+        <is>
+          <t>Brighton; Programme — programme held; abstract book available — ask Cat</t>
+        </is>
+      </c>
+      <c r="E109" s="13" t="inlineStr"/>
+      <c r="F109" s="13" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" s="10" t="n">
+      <c r="A110" s="11" t="n">
         <v>2024</v>
       </c>
-      <c r="B110" s="16" t="inlineStr">
-        <is>
-          <t>Pittsburgh, PA; Schedule</t>
-        </is>
-      </c>
-      <c r="C110" s="16" t="inlineStr">
-        <is>
-          <t>Pittsburgh, PA (97); Schedule</t>
+      <c r="B110" s="17" t="inlineStr">
+        <is>
+          <t>Pittsburgh, PA; Schedule — programme ingested (no abstract bodies)</t>
+        </is>
+      </c>
+      <c r="C110" s="17" t="inlineStr">
+        <is>
+          <t>Pittsburgh, PA (97); Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
       <c r="D110" s="18" t="inlineStr">
         <is>
-          <t>Thessaloniki; Digital</t>
-        </is>
-      </c>
-      <c r="E110" s="17" t="inlineStr">
-        <is>
-          <t>?; Pending (Brit)</t>
-        </is>
-      </c>
-      <c r="F110" s="12" t="inlineStr"/>
+          <t>Thessaloniki; Pending — abstract book available — ask Cat</t>
+        </is>
+      </c>
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Brit collating (council approval)</t>
+        </is>
+      </c>
+      <c r="F110" s="13" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" s="10" t="n">
+      <c r="A111" s="11" t="n">
         <v>2025</v>
       </c>
-      <c r="B111" s="16" t="inlineStr">
-        <is>
-          <t>St. Paul, MN; Schedule</t>
-        </is>
-      </c>
-      <c r="C111" s="16" t="inlineStr">
-        <is>
-          <t>St. Paul, MN (68); Schedule</t>
+      <c r="B111" s="17" t="inlineStr">
+        <is>
+          <t>St. Paul, MN; Schedule — programme ingested (no abstract bodies)</t>
+        </is>
+      </c>
+      <c r="C111" s="17" t="inlineStr">
+        <is>
+          <t>St. Paul, MN (68); Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
       <c r="D111" s="18" t="inlineStr">
         <is>
-          <t>Rotterdam; Digital</t>
-        </is>
-      </c>
-      <c r="E111" s="12" t="inlineStr"/>
-      <c r="F111" s="12" t="inlineStr"/>
+          <t>Rotterdam; Pending — abstract book available — ask Cat</t>
+        </is>
+      </c>
+      <c r="E111" s="13" t="inlineStr"/>
+      <c r="F111" s="13" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" s="10" t="n">
+      <c r="A112" s="11" t="n">
         <v>2026</v>
       </c>
-      <c r="B112" s="18" t="inlineStr">
-        <is>
-          <t>New Orleans, LA; Digital</t>
-        </is>
-      </c>
-      <c r="C112" s="18" t="inlineStr">
-        <is>
-          <t>New Orleans, LA; Digital</t>
+      <c r="B112" s="20" t="inlineStr">
+        <is>
+          <t>New Orleans, LA; Programme — image-only programme — needs OCR; abstract book needed</t>
+        </is>
+      </c>
+      <c r="C112" s="20" t="inlineStr">
+        <is>
+          <t>New Orleans, LA; Programme — image-only programme — needs OCR; abstract book needed</t>
         </is>
       </c>
       <c r="D112" s="18" t="inlineStr">
         <is>
-          <t>online; Digital</t>
-        </is>
-      </c>
-      <c r="E112" s="17" t="inlineStr">
-        <is>
-          <t>?; Pending (Brit)</t>
-        </is>
-      </c>
-      <c r="F112" s="15" t="inlineStr">
+          <t>online; Pending — will be digital</t>
+        </is>
+      </c>
+      <c r="E112" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Brit collating (council approval)</t>
+        </is>
+      </c>
+      <c r="F112" s="16" t="inlineStr">
         <is>
           <t>Colombo; Ingested</t>
         </is>
@@ -3098,7 +3120,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Conference abstract coverage — dashboard</t>
         </is>

</xml_diff>

<commit_message>
docs(conf-abstracts): mark EEA 2004-2019 + 2023 Ingested in coverage matrix
Fable extraction complete (731 abstracts). EEA column now shows Ingested with
per-book counts for 2004/2011/2013/2014/2016/2017/2018/2019/2023; 2015 =
Programme (2-page, 0 abstracts); 2024/2025 = Pending (PDFs corrupt, await clean
copies from Cat). Guard confirmed no colleague edits before rebuild; schema clean.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -121,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -155,9 +155,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1121,7 +1118,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>- EEA 2010-2026 from Cat Gordon (Shark Trust); pre-2010 in Ali's archive. EEA not yet ingested. SI2022 Valencia PDF received (Digital).</t>
+          <t>- EEA 2010-2026 from Cat Gordon (Shark Trust); pre-2010 in Ali's archive. EEA 2004-2019 + 2023 ingested via Fable (731 abstracts, 2026-08-14); 2024/2025 PDFs corrupt (await clean copies from Cat). SI2022 Valencia PDF received (Digital).</t>
         </is>
       </c>
     </row>
@@ -2558,9 +2555,9 @@
           <t>Norman, OK; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D90" s="14" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D90" s="16" t="inlineStr">
+        <is>
+          <t>London; Ingested — 55 abstracts (Fable)</t>
         </is>
       </c>
       <c r="E90" s="13" t="inlineStr"/>
@@ -2716,9 +2713,9 @@
           <t>Minneapolis, MN; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D97" s="14" t="inlineStr">
-        <is>
-          <t>Berlin; Hardcopy — Cat has hardcopy</t>
+      <c r="D97" s="16" t="inlineStr">
+        <is>
+          <t>Berlin; Ingested — 58 abstracts (Fable)</t>
         </is>
       </c>
       <c r="E97" s="13" t="inlineStr"/>
@@ -2764,9 +2761,9 @@
           <t>Albuquerque, NM; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D99" s="19" t="inlineStr">
-        <is>
-          <t>Plymouth; Digital — abstract book held — ingest</t>
+      <c r="D99" s="16" t="inlineStr">
+        <is>
+          <t>Plymouth; Ingested — 93 abstracts (Fable)</t>
         </is>
       </c>
       <c r="E99" s="13" t="inlineStr"/>
@@ -2786,9 +2783,9 @@
           <t>Chattanooga, TN; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D100" s="14" t="inlineStr">
-        <is>
-          <t>Leeuwarden; Hardcopy — Cat has hardcopy</t>
+      <c r="D100" s="16" t="inlineStr">
+        <is>
+          <t>Leeuwarden; Ingested — 61 abstracts (Fable)</t>
         </is>
       </c>
       <c r="E100" s="18" t="inlineStr">
@@ -2818,7 +2815,7 @@
       </c>
       <c r="D101" s="19" t="inlineStr">
         <is>
-          <t>Peniche; Digital — abstract book held — ingest</t>
+          <t>Peniche; Programme — 2-page programme only (0 abstracts) — abstract book needed</t>
         </is>
       </c>
       <c r="E101" s="13" t="inlineStr"/>
@@ -2838,9 +2835,9 @@
           <t>New Orleans, LA (240); Ingested</t>
         </is>
       </c>
-      <c r="D102" s="14" t="inlineStr">
-        <is>
-          <t>Bristol; Hardcopy — Cat (Shark Trust) hosted — ask for print PDF</t>
+      <c r="D102" s="16" t="inlineStr">
+        <is>
+          <t>Bristol; Ingested — 93 abstracts (Fable)</t>
         </is>
       </c>
       <c r="E102" s="18" t="inlineStr">
@@ -2854,19 +2851,19 @@
       <c r="A103" s="11" t="n">
         <v>2017</v>
       </c>
-      <c r="B103" s="20" t="inlineStr">
+      <c r="B103" s="19" t="inlineStr">
         <is>
           <t>Austin, TX; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
       </c>
-      <c r="C103" s="20" t="inlineStr">
+      <c r="C103" s="19" t="inlineStr">
         <is>
           <t>Austin, TX; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
       </c>
-      <c r="D103" s="20" t="inlineStr">
-        <is>
-          <t>Amsterdam; Programme — only programme held — abstract book needed</t>
+      <c r="D103" s="16" t="inlineStr">
+        <is>
+          <t>Amsterdam; Ingested — 62 talks, programme/no bodies (Fable)</t>
         </is>
       </c>
       <c r="E103" s="13" t="inlineStr"/>
@@ -2886,9 +2883,9 @@
           <t>Rochester, NY; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D104" s="12" t="inlineStr">
-        <is>
-          <t>Peniche; Missing — Cat: no hardcopy, likely online-only — find</t>
+      <c r="D104" s="16" t="inlineStr">
+        <is>
+          <t>Peniche; Ingested — 75 abstracts (Fable)</t>
         </is>
       </c>
       <c r="E104" s="18" t="inlineStr">
@@ -2906,19 +2903,19 @@
       <c r="A105" s="11" t="n">
         <v>2019</v>
       </c>
-      <c r="B105" s="20" t="inlineStr">
+      <c r="B105" s="19" t="inlineStr">
         <is>
           <t>Snowbird, UT; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
       </c>
-      <c r="C105" s="20" t="inlineStr">
+      <c r="C105" s="19" t="inlineStr">
         <is>
           <t>Snowbird, UT; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
       </c>
-      <c r="D105" s="14" t="inlineStr">
-        <is>
-          <t>Rende; Hardcopy — Cat has hardcopy</t>
+      <c r="D105" s="16" t="inlineStr">
+        <is>
+          <t>Rende; Ingested — 136 abstracts (Fable)</t>
         </is>
       </c>
       <c r="E105" s="13" t="inlineStr"/>
@@ -2964,7 +2961,7 @@
           <t>Phoenix, AZ (46); Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
-      <c r="D107" s="20" t="inlineStr">
+      <c r="D107" s="19" t="inlineStr">
         <is>
           <t>Leiden; Programme — only programme held — abstract book needed</t>
         </is>
@@ -3016,9 +3013,9 @@
           <t>Norfolk, VA (87); Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
-      <c r="D109" s="20" t="inlineStr">
-        <is>
-          <t>Brighton; Programme — programme held; abstract book available — ask Cat</t>
+      <c r="D109" s="16" t="inlineStr">
+        <is>
+          <t>Brighton; Ingested — oral 64 + poster 34 = 98 abstracts (Fable)</t>
         </is>
       </c>
       <c r="E109" s="13" t="inlineStr"/>
@@ -3040,7 +3037,7 @@
       </c>
       <c r="D110" s="18" t="inlineStr">
         <is>
-          <t>Thessaloniki; Pending — abstract book available — ask Cat</t>
+          <t>Thessaloniki; Pending — PDF corrupt — need clean copy from Cat</t>
         </is>
       </c>
       <c r="E110" s="18" t="inlineStr">
@@ -3066,7 +3063,7 @@
       </c>
       <c r="D111" s="18" t="inlineStr">
         <is>
-          <t>Rotterdam; Pending — abstract book available — ask Cat</t>
+          <t>Rotterdam; Pending — PDF corrupt — need clean copy from Cat</t>
         </is>
       </c>
       <c r="E111" s="13" t="inlineStr"/>
@@ -3076,12 +3073,12 @@
       <c r="A112" s="11" t="n">
         <v>2026</v>
       </c>
-      <c r="B112" s="20" t="inlineStr">
+      <c r="B112" s="19" t="inlineStr">
         <is>
           <t>New Orleans, LA; Programme — image-only programme — needs OCR; abstract book needed</t>
         </is>
       </c>
-      <c r="C112" s="20" t="inlineStr">
+      <c r="C112" s="19" t="inlineStr">
         <is>
           <t>New Orleans, LA; Programme — image-only programme — needs OCR; abstract book needed</t>
         </is>
@@ -3120,7 +3117,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Conference abstract coverage — dashboard</t>
         </is>

</xml_diff>

<commit_message>
fix(conf-abstracts): content-aware coverage matrix — 2008 JMIH Ingested, 2003/2004 OCR-failed, 2026 note
- builder: LEFT JOIN meetings so held-but-unparsed books surface; treat a
  'programme' whose records carry bodies as an abstract book; new OCR-failed
  state for degraded scans that yielded 0 records (JMIH 2003/2004).
- classifier: 200+ page 'programme' PDFs are abstract books (2008 JMIH.pdf,
  520pp, 585 abstracts); DB row 12 doc_type corrected.
- 2026 JMIH programme already has an OCR text layer; note corrected.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -151,13 +151,13 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2523,14 +2523,14 @@
       <c r="A89" s="11" t="n">
         <v>2003</v>
       </c>
-      <c r="B89" s="14" t="inlineStr">
-        <is>
-          <t>Manaus, Brazil; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
-        </is>
-      </c>
-      <c r="C89" s="14" t="inlineStr">
-        <is>
-          <t>Manaus, Brazil; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+      <c r="B89" s="15" t="inlineStr">
+        <is>
+          <t>Manaus, Brazil; OCR — degraded phone scan — 0 abstracts recovered — flatbed re-scan needed (Carylanne)</t>
+        </is>
+      </c>
+      <c r="C89" s="15" t="inlineStr">
+        <is>
+          <t>Manaus, Brazil; OCR — degraded phone scan — 0 abstracts recovered — flatbed re-scan needed (Carylanne)</t>
         </is>
       </c>
       <c r="D89" s="14" t="inlineStr">
@@ -2545,14 +2545,14 @@
       <c r="A90" s="11" t="n">
         <v>2004</v>
       </c>
-      <c r="B90" s="14" t="inlineStr">
-        <is>
-          <t>Norman, OK; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
-        </is>
-      </c>
-      <c r="C90" s="14" t="inlineStr">
-        <is>
-          <t>Norman, OK; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+      <c r="B90" s="15" t="inlineStr">
+        <is>
+          <t>Norman, OK; OCR — degraded phone scan — 0 abstracts recovered — flatbed re-scan needed (Carylanne)</t>
+        </is>
+      </c>
+      <c r="C90" s="15" t="inlineStr">
+        <is>
+          <t>Norman, OK; OCR — degraded phone scan — 0 abstracts recovered — flatbed re-scan needed (Carylanne)</t>
         </is>
       </c>
       <c r="D90" s="16" t="inlineStr">
@@ -2633,14 +2633,14 @@
       <c r="A94" s="11" t="n">
         <v>2008</v>
       </c>
-      <c r="B94" s="17" t="inlineStr">
-        <is>
-          <t>Montreal, PQ; Schedule — programme ingested (no abstract bodies)</t>
-        </is>
-      </c>
-      <c r="C94" s="17" t="inlineStr">
-        <is>
-          <t>Montreal, PQ (193); Schedule — programme ingested (no abstract bodies)</t>
+      <c r="B94" s="16" t="inlineStr">
+        <is>
+          <t>Montreal, PQ; Ingested</t>
+        </is>
+      </c>
+      <c r="C94" s="16" t="inlineStr">
+        <is>
+          <t>Montreal, PQ (193); Ingested</t>
         </is>
       </c>
       <c r="D94" s="14" t="inlineStr">
@@ -2740,7 +2740,7 @@
           <t>Milan; Hardcopy — Cat has hardcopy</t>
         </is>
       </c>
-      <c r="E98" s="18" t="inlineStr">
+      <c r="E98" s="17" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -2788,7 +2788,7 @@
           <t>Leeuwarden; Ingested — 61 abstracts (Fable)</t>
         </is>
       </c>
-      <c r="E100" s="18" t="inlineStr">
+      <c r="E100" s="17" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -2813,7 +2813,7 @@
           <t>Reno, NV (123); Ingested</t>
         </is>
       </c>
-      <c r="D101" s="19" t="inlineStr">
+      <c r="D101" s="18" t="inlineStr">
         <is>
           <t>Peniche; Programme — 2-page programme only (0 abstracts) — abstract book needed</t>
         </is>
@@ -2840,7 +2840,7 @@
           <t>Bristol; Ingested — 93 abstracts (Fable)</t>
         </is>
       </c>
-      <c r="E102" s="18" t="inlineStr">
+      <c r="E102" s="17" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -2851,12 +2851,12 @@
       <c r="A103" s="11" t="n">
         <v>2017</v>
       </c>
-      <c r="B103" s="19" t="inlineStr">
+      <c r="B103" s="18" t="inlineStr">
         <is>
           <t>Austin, TX; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
       </c>
-      <c r="C103" s="19" t="inlineStr">
+      <c r="C103" s="18" t="inlineStr">
         <is>
           <t>Austin, TX; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
@@ -2888,7 +2888,7 @@
           <t>Peniche; Ingested — 75 abstracts (Fable)</t>
         </is>
       </c>
-      <c r="E104" s="18" t="inlineStr">
+      <c r="E104" s="17" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -2903,12 +2903,12 @@
       <c r="A105" s="11" t="n">
         <v>2019</v>
       </c>
-      <c r="B105" s="19" t="inlineStr">
+      <c r="B105" s="18" t="inlineStr">
         <is>
           <t>Snowbird, UT; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
       </c>
-      <c r="C105" s="19" t="inlineStr">
+      <c r="C105" s="18" t="inlineStr">
         <is>
           <t>Snowbird, UT; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
@@ -2940,7 +2940,7 @@
           <t>online (covid); Missing — covid/online — find</t>
         </is>
       </c>
-      <c r="E106" s="18" t="inlineStr">
+      <c r="E106" s="17" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -2951,17 +2951,17 @@
       <c r="A107" s="11" t="n">
         <v>2021</v>
       </c>
-      <c r="B107" s="17" t="inlineStr">
+      <c r="B107" s="19" t="inlineStr">
         <is>
           <t>Phoenix, AZ; Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
-      <c r="C107" s="17" t="inlineStr">
+      <c r="C107" s="19" t="inlineStr">
         <is>
           <t>Phoenix, AZ (46); Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
-      <c r="D107" s="19" t="inlineStr">
+      <c r="D107" s="18" t="inlineStr">
         <is>
           <t>Leiden; Programme — only programme held — abstract book needed</t>
         </is>
@@ -2973,27 +2973,27 @@
       <c r="A108" s="11" t="n">
         <v>2022</v>
       </c>
-      <c r="B108" s="17" t="inlineStr">
+      <c r="B108" s="19" t="inlineStr">
         <is>
           <t>Spokane, WA; Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
-      <c r="C108" s="17" t="inlineStr">
+      <c r="C108" s="19" t="inlineStr">
         <is>
           <t>Spokane, WA (69); Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
-      <c r="D108" s="17" t="inlineStr">
+      <c r="D108" s="19" t="inlineStr">
         <is>
           <t>Valencia (=SI2022); Schedule — covered via SI2022 (schedule)</t>
         </is>
       </c>
-      <c r="E108" s="18" t="inlineStr">
+      <c r="E108" s="17" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
       </c>
-      <c r="F108" s="17" t="inlineStr">
+      <c r="F108" s="19" t="inlineStr">
         <is>
           <t>Valencia; Schedule — programme ingested (no bodies)</t>
         </is>
@@ -3003,12 +3003,12 @@
       <c r="A109" s="11" t="n">
         <v>2023</v>
       </c>
-      <c r="B109" s="17" t="inlineStr">
+      <c r="B109" s="19" t="inlineStr">
         <is>
           <t>Norfolk, VA; Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
-      <c r="C109" s="17" t="inlineStr">
+      <c r="C109" s="19" t="inlineStr">
         <is>
           <t>Norfolk, VA (87); Schedule — programme ingested (no abstract bodies)</t>
         </is>
@@ -3025,22 +3025,22 @@
       <c r="A110" s="11" t="n">
         <v>2024</v>
       </c>
-      <c r="B110" s="17" t="inlineStr">
+      <c r="B110" s="19" t="inlineStr">
         <is>
           <t>Pittsburgh, PA; Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
-      <c r="C110" s="17" t="inlineStr">
+      <c r="C110" s="19" t="inlineStr">
         <is>
           <t>Pittsburgh, PA (97); Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
-      <c r="D110" s="18" t="inlineStr">
+      <c r="D110" s="17" t="inlineStr">
         <is>
           <t>Thessaloniki; Pending — PDF corrupt — need clean copy from Cat</t>
         </is>
       </c>
-      <c r="E110" s="18" t="inlineStr">
+      <c r="E110" s="17" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -3051,17 +3051,17 @@
       <c r="A111" s="11" t="n">
         <v>2025</v>
       </c>
-      <c r="B111" s="17" t="inlineStr">
+      <c r="B111" s="19" t="inlineStr">
         <is>
           <t>St. Paul, MN; Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
-      <c r="C111" s="17" t="inlineStr">
+      <c r="C111" s="19" t="inlineStr">
         <is>
           <t>St. Paul, MN (68); Schedule — programme ingested (no abstract bodies)</t>
         </is>
       </c>
-      <c r="D111" s="18" t="inlineStr">
+      <c r="D111" s="17" t="inlineStr">
         <is>
           <t>Rotterdam; Pending — PDF corrupt — need clean copy from Cat</t>
         </is>
@@ -3073,22 +3073,22 @@
       <c r="A112" s="11" t="n">
         <v>2026</v>
       </c>
-      <c r="B112" s="19" t="inlineStr">
-        <is>
-          <t>New Orleans, LA; Programme — image-only programme — needs OCR; abstract book needed</t>
-        </is>
-      </c>
-      <c r="C112" s="19" t="inlineStr">
-        <is>
-          <t>New Orleans, LA; Programme — image-only programme — needs OCR; abstract book needed</t>
-        </is>
-      </c>
-      <c r="D112" s="18" t="inlineStr">
+      <c r="B112" s="18" t="inlineStr">
+        <is>
+          <t>New Orleans, LA; Programme — schedule-only programme (OCR text layer OK, not yet parsed) — abstract book needed</t>
+        </is>
+      </c>
+      <c r="C112" s="18" t="inlineStr">
+        <is>
+          <t>New Orleans, LA; Programme — schedule-only programme (OCR text layer OK, not yet parsed) — abstract book needed</t>
+        </is>
+      </c>
+      <c r="D112" s="17" t="inlineStr">
         <is>
           <t>online; Pending — will be digital</t>
         </is>
       </c>
-      <c r="E112" s="18" t="inlineStr">
+      <c r="E112" s="17" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>

</xml_diff>

<commit_message>
feat(conf-abstracts): harvest AES 1985-2005 from elasmo.org; one DB of record; library migration
- scrape_elasmo_org.py: 21 AES annual-meeting pages (full bodies) -> 1,305
  abstracts; --dedup/--supersede remove the JMIH-book copies of the same AES
  talks (degraded 1997-2001 OCR and the 2005 A3 parse).
- merge_fable_into_main.py: Fable-extracted EEA books (731) folded into
  conference_abstracts.db, which is now the single DB of record (11,487
  abstracts / 4,869 elasmo). Exports refreshed beside both DBs.
- Conference PDFs renamed YYYY_<Conf>_<Type>[_qualifier].pdf and copied to
  SharkPapers/Conferences/YYYY/ (pathmap json); DB source_pdf repointed;
  config/run_pipeline/classify/conf_fable_prep follow the new tree.
  others_libraries/{Carylanne,Cat} stay as partner inboxes.
- coverage matrix: AES column from elasmo.org, EEA on the dashboard,
  Schedule cells say the abstract book is still needed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -142,13 +142,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -269,12 +269,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$B$3:$G$3</f>
+              <f>'Dashboard'!$B$3:$H$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$B$39:$G$39</f>
+              <f>'Dashboard'!$B$39:$H$39</f>
             </numRef>
           </val>
         </ser>
@@ -536,6 +536,38 @@
           <val>
             <numRef>
               <f>'Dashboard'!$G$4:$G$38</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!H3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$4:$A$38</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$H$4:$H$38</f>
             </numRef>
           </val>
         </ser>
@@ -942,7 +974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1104,40 +1136,47 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>- 'OCR' = degraded 1997-2004 JMIH phone-photo scans (all needs_review); Carylanne's flatbed re-scans will upgrade these.</t>
+          <t>- 'OCR' = degraded 1997-2004 JMIH phone-photo scans (all needs_review); Carylanne's flatbed re-scans would upgrade the non-AES content.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>- No abstracts collected pre-1992 (Carylanne's archive starts 1992) → 1916-1991 show host city but 'Missing'.</t>
+          <t>- AES 1985-2005: full abstracts harvested from elasmo.org/meetings/abstracts/abst&lt;YYYY&gt;/ (1,305 abstracts, 2026-08-25); JMIH-book copies of the same AES talks were removed. No AES source found for 1983-84 or 2006+ online.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>- EEA 2010-2026 from Cat Gordon (Shark Trust); pre-2010 in Ali's archive. EEA 2004-2019 + 2023 ingested via Fable (731 abstracts, 2026-08-14); 2024/2025 PDFs corrupt (await clean copies from Cat). SI2022 Valencia PDF received (Digital).</t>
+          <t>- ASIH/JMIH pre-1992: Carylanne's archive starts 1992 → host city shown but 'Missing'.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>- OCS (Oceania Chondrichthyan Soc, ~2011+, biennial): Brit Finucci collating, pending council — years/locations TBC.</t>
+          <t>- EEA 2010-2026 from Cat Gordon (Shark Trust); pre-2010 in Ali's archive. EEA 2004-2019 + 2023 ingested via Fable (731 abstracts, 2026-08-14) and merged into the main DB 2026-08-25; 2024/2025 PDFs corrupt (await clean copies from Cat). SI2022 Valencia schedule ingested.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>- Blank/unshaded cell = no conference that year for that series.</t>
+          <t>- OCS (Oceania Chondrichthyan Soc, ~2011+, biennial): Brit Finucci collating, pending council — years/locations TBC.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
+        <is>
+          <t>- Blank/unshaded cell = no conference that year for that series.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>- Per-society counts &amp; trends: see the Dashboard tab.</t>
         </is>
@@ -2180,9 +2219,9 @@
           <t>Knoxville, TN; Missing</t>
         </is>
       </c>
-      <c r="C71" s="12" t="inlineStr">
-        <is>
-          <t>Knoxville, TN; Missing</t>
+      <c r="C71" s="14" t="inlineStr">
+        <is>
+          <t>Knoxville, TN (26); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr"/>
@@ -2198,9 +2237,9 @@
           <t>Victoria, BC; Missing</t>
         </is>
       </c>
-      <c r="C72" s="12" t="inlineStr">
-        <is>
-          <t>Victoria, BC; Missing</t>
+      <c r="C72" s="14" t="inlineStr">
+        <is>
+          <t>Victoria, BC (35); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr"/>
@@ -2216,9 +2255,9 @@
           <t>Albany, NY; Missing</t>
         </is>
       </c>
-      <c r="C73" s="12" t="inlineStr">
-        <is>
-          <t>Albany, NY; Missing</t>
+      <c r="C73" s="14" t="inlineStr">
+        <is>
+          <t>Albany, NY (33); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D73" s="13" t="inlineStr"/>
@@ -2234,9 +2273,9 @@
           <t>Ann Arbor, MI; Missing</t>
         </is>
       </c>
-      <c r="C74" s="12" t="inlineStr">
-        <is>
-          <t>Ann Arbor, MI; Missing</t>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>Ann Arbor, MI (34); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D74" s="13" t="inlineStr"/>
@@ -2252,9 +2291,9 @@
           <t>San Francisco, CA; Missing</t>
         </is>
       </c>
-      <c r="C75" s="12" t="inlineStr">
-        <is>
-          <t>San Francisco, CA; Missing</t>
+      <c r="C75" s="14" t="inlineStr">
+        <is>
+          <t>San Francisco, CA (63); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D75" s="13" t="inlineStr"/>
@@ -2270,9 +2309,9 @@
           <t>Charleston, SC; Missing</t>
         </is>
       </c>
-      <c r="C76" s="12" t="inlineStr">
-        <is>
-          <t>Charleston, SC; Missing</t>
+      <c r="C76" s="14" t="inlineStr">
+        <is>
+          <t>Charleston, SC (47); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D76" s="13" t="inlineStr"/>
@@ -2288,9 +2327,9 @@
           <t>New York, NY; Missing</t>
         </is>
       </c>
-      <c r="C77" s="12" t="inlineStr">
-        <is>
-          <t>New York, NY; Missing</t>
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>New York, NY (34); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D77" s="13" t="inlineStr"/>
@@ -2301,14 +2340,14 @@
       <c r="A78" s="11" t="n">
         <v>1992</v>
       </c>
-      <c r="B78" s="14" t="inlineStr">
+      <c r="B78" s="15" t="inlineStr">
         <is>
           <t>Champaign-Urbana, IL; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
       <c r="C78" s="14" t="inlineStr">
         <is>
-          <t>Champaign-Urbana, IL; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+          <t>Champaign-Urbana, IL (41); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D78" s="13" t="inlineStr"/>
@@ -2319,14 +2358,14 @@
       <c r="A79" s="11" t="n">
         <v>1993</v>
       </c>
-      <c r="B79" s="14" t="inlineStr">
+      <c r="B79" s="15" t="inlineStr">
         <is>
           <t>Austin, TX; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
       <c r="C79" s="14" t="inlineStr">
         <is>
-          <t>Austin, TX; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+          <t>Austin, TX (45); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D79" s="13" t="inlineStr"/>
@@ -2337,14 +2376,14 @@
       <c r="A80" s="11" t="n">
         <v>1994</v>
       </c>
-      <c r="B80" s="14" t="inlineStr">
+      <c r="B80" s="15" t="inlineStr">
         <is>
           <t>Los Angeles, CA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
       <c r="C80" s="14" t="inlineStr">
         <is>
-          <t>Los Angeles, CA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+          <t>Los Angeles, CA (50); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D80" s="13" t="inlineStr"/>
@@ -2355,14 +2394,14 @@
       <c r="A81" s="11" t="n">
         <v>1995</v>
       </c>
-      <c r="B81" s="14" t="inlineStr">
+      <c r="B81" s="15" t="inlineStr">
         <is>
           <t>Edmonton, AB; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
       <c r="C81" s="14" t="inlineStr">
         <is>
-          <t>Edmonton, AB; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+          <t>Edmonton, AB (46); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D81" s="13" t="inlineStr"/>
@@ -2373,14 +2412,14 @@
       <c r="A82" s="11" t="n">
         <v>1996</v>
       </c>
-      <c r="B82" s="14" t="inlineStr">
+      <c r="B82" s="15" t="inlineStr">
         <is>
           <t>New Orleans, LA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
       <c r="C82" s="14" t="inlineStr">
         <is>
-          <t>New Orleans, LA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
+          <t>New Orleans, LA (98); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
       <c r="D82" s="13" t="inlineStr"/>
@@ -2391,17 +2430,17 @@
       <c r="A83" s="11" t="n">
         <v>1997</v>
       </c>
-      <c r="B83" s="15" t="inlineStr">
+      <c r="B83" s="16" t="inlineStr">
         <is>
           <t>Seattle, WA; OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
         </is>
       </c>
-      <c r="C83" s="15" t="inlineStr">
-        <is>
-          <t>Seattle, WA (58); OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
-        </is>
-      </c>
-      <c r="D83" s="14" t="inlineStr">
+      <c r="C83" s="14" t="inlineStr">
+        <is>
+          <t>Seattle, WA (68); Ingested — AES abstracts from elasmo.org (full bodies)</t>
+        </is>
+      </c>
+      <c r="D83" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2413,17 +2452,17 @@
       <c r="A84" s="11" t="n">
         <v>1998</v>
       </c>
-      <c r="B84" s="15" t="inlineStr">
+      <c r="B84" s="16" t="inlineStr">
         <is>
           <t>Guelph, ON; OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
         </is>
       </c>
-      <c r="C84" s="15" t="inlineStr">
-        <is>
-          <t>Guelph, ON (15); OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
-        </is>
-      </c>
-      <c r="D84" s="14" t="inlineStr">
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>Guelph, ON (63); Ingested — AES abstracts from elasmo.org (full bodies)</t>
+        </is>
+      </c>
+      <c r="D84" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2435,17 +2474,17 @@
       <c r="A85" s="11" t="n">
         <v>1999</v>
       </c>
-      <c r="B85" s="15" t="inlineStr">
+      <c r="B85" s="16" t="inlineStr">
         <is>
           <t>University Park, PA; OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
         </is>
       </c>
-      <c r="C85" s="15" t="inlineStr">
-        <is>
-          <t>University Park, PA (57); OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
-        </is>
-      </c>
-      <c r="D85" s="14" t="inlineStr">
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>University Park, PA (78); Ingested — AES abstracts from elasmo.org (full bodies)</t>
+        </is>
+      </c>
+      <c r="D85" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2457,17 +2496,17 @@
       <c r="A86" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="B86" s="15" t="inlineStr">
+      <c r="B86" s="16" t="inlineStr">
         <is>
           <t>La Paz, Mexico; OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
         </is>
       </c>
-      <c r="C86" s="15" t="inlineStr">
-        <is>
-          <t>La Paz, Mexico (59); OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
-        </is>
-      </c>
-      <c r="D86" s="14" t="inlineStr">
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>La Paz, Mexico (134); Ingested — AES abstracts from elasmo.org (full bodies)</t>
+        </is>
+      </c>
+      <c r="D86" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2479,17 +2518,17 @@
       <c r="A87" s="11" t="n">
         <v>2001</v>
       </c>
-      <c r="B87" s="15" t="inlineStr">
+      <c r="B87" s="16" t="inlineStr">
         <is>
           <t>University Park, PA; OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
         </is>
       </c>
-      <c r="C87" s="15" t="inlineStr">
-        <is>
-          <t>University Park, PA (67); OCR — degraded scan (needs_review) — flatbed re-scan planned</t>
-        </is>
-      </c>
-      <c r="D87" s="14" t="inlineStr">
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>University Park, PA (84); Ingested — AES abstracts from elasmo.org (full bodies)</t>
+        </is>
+      </c>
+      <c r="D87" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2501,17 +2540,17 @@
       <c r="A88" s="11" t="n">
         <v>2002</v>
       </c>
-      <c r="B88" s="14" t="inlineStr">
+      <c r="B88" s="15" t="inlineStr">
         <is>
           <t>Kansas City, MO; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
       <c r="C88" s="14" t="inlineStr">
         <is>
-          <t>Kansas City, MO; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
-        </is>
-      </c>
-      <c r="D88" s="14" t="inlineStr">
+          <t>Kansas City, MO (27); Ingested — AES abstracts from elasmo.org (full bodies)</t>
+        </is>
+      </c>
+      <c r="D88" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2523,17 +2562,17 @@
       <c r="A89" s="11" t="n">
         <v>2003</v>
       </c>
-      <c r="B89" s="15" t="inlineStr">
+      <c r="B89" s="16" t="inlineStr">
         <is>
           <t>Manaus, Brazil; OCR — degraded phone scan — 0 abstracts recovered — flatbed re-scan needed (Carylanne)</t>
         </is>
       </c>
-      <c r="C89" s="15" t="inlineStr">
-        <is>
-          <t>Manaus, Brazil; OCR — degraded phone scan — 0 abstracts recovered — flatbed re-scan needed (Carylanne)</t>
-        </is>
-      </c>
-      <c r="D89" s="14" t="inlineStr">
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>Manaus, Brazil (82); Ingested — AES abstracts from elasmo.org (full bodies)</t>
+        </is>
+      </c>
+      <c r="D89" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2545,17 +2584,17 @@
       <c r="A90" s="11" t="n">
         <v>2004</v>
       </c>
-      <c r="B90" s="15" t="inlineStr">
+      <c r="B90" s="16" t="inlineStr">
         <is>
           <t>Norman, OK; OCR — degraded phone scan — 0 abstracts recovered — flatbed re-scan needed (Carylanne)</t>
         </is>
       </c>
-      <c r="C90" s="15" t="inlineStr">
-        <is>
-          <t>Norman, OK; OCR — degraded phone scan — 0 abstracts recovered — flatbed re-scan needed (Carylanne)</t>
-        </is>
-      </c>
-      <c r="D90" s="16" t="inlineStr">
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>Norman, OK (59); Ingested — AES abstracts from elasmo.org (full bodies)</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
         <is>
           <t>London; Ingested — 55 abstracts (Fable)</t>
         </is>
@@ -2567,17 +2606,17 @@
       <c r="A91" s="11" t="n">
         <v>2005</v>
       </c>
-      <c r="B91" s="16" t="inlineStr">
+      <c r="B91" s="14" t="inlineStr">
         <is>
           <t>Tampa, FL; Ingested</t>
         </is>
       </c>
-      <c r="C91" s="16" t="inlineStr">
-        <is>
-          <t>Tampa, FL (80); Ingested</t>
-        </is>
-      </c>
-      <c r="D91" s="14" t="inlineStr">
+      <c r="C91" s="14" t="inlineStr">
+        <is>
+          <t>Tampa, FL (158); Ingested — AES abstracts from elasmo.org (full bodies)</t>
+        </is>
+      </c>
+      <c r="D91" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2589,17 +2628,17 @@
       <c r="A92" s="11" t="n">
         <v>2006</v>
       </c>
-      <c r="B92" s="14" t="inlineStr">
+      <c r="B92" s="15" t="inlineStr">
         <is>
           <t>New Orleans, LA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="C92" s="14" t="inlineStr">
+      <c r="C92" s="15" t="inlineStr">
         <is>
           <t>New Orleans, LA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D92" s="14" t="inlineStr">
+      <c r="D92" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2611,17 +2650,17 @@
       <c r="A93" s="11" t="n">
         <v>2007</v>
       </c>
-      <c r="B93" s="16" t="inlineStr">
+      <c r="B93" s="14" t="inlineStr">
         <is>
           <t>St. Louis, MO; Ingested</t>
         </is>
       </c>
-      <c r="C93" s="16" t="inlineStr">
+      <c r="C93" s="14" t="inlineStr">
         <is>
           <t>St. Louis, MO (155); Ingested</t>
         </is>
       </c>
-      <c r="D93" s="14" t="inlineStr">
+      <c r="D93" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2633,17 +2672,17 @@
       <c r="A94" s="11" t="n">
         <v>2008</v>
       </c>
-      <c r="B94" s="16" t="inlineStr">
+      <c r="B94" s="14" t="inlineStr">
         <is>
           <t>Montreal, PQ; Ingested</t>
         </is>
       </c>
-      <c r="C94" s="16" t="inlineStr">
+      <c r="C94" s="14" t="inlineStr">
         <is>
           <t>Montreal, PQ (193); Ingested</t>
         </is>
       </c>
-      <c r="D94" s="14" t="inlineStr">
+      <c r="D94" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2655,17 +2694,17 @@
       <c r="A95" s="11" t="n">
         <v>2009</v>
       </c>
-      <c r="B95" s="16" t="inlineStr">
+      <c r="B95" s="14" t="inlineStr">
         <is>
           <t>Portland, OR; Ingested</t>
         </is>
       </c>
-      <c r="C95" s="16" t="inlineStr">
+      <c r="C95" s="14" t="inlineStr">
         <is>
           <t>Portland, OR (149); Ingested</t>
         </is>
       </c>
-      <c r="D95" s="14" t="inlineStr">
+      <c r="D95" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
         </is>
@@ -2677,17 +2716,17 @@
       <c r="A96" s="11" t="n">
         <v>2010</v>
       </c>
-      <c r="B96" s="14" t="inlineStr">
+      <c r="B96" s="15" t="inlineStr">
         <is>
           <t>Providence, RI; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="C96" s="14" t="inlineStr">
+      <c r="C96" s="15" t="inlineStr">
         <is>
           <t>Providence, RI; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D96" s="14" t="inlineStr">
+      <c r="D96" s="15" t="inlineStr">
         <is>
           <t>Galway; Hardcopy — Cat has hardcopy</t>
         </is>
@@ -2703,17 +2742,17 @@
       <c r="A97" s="11" t="n">
         <v>2011</v>
       </c>
-      <c r="B97" s="14" t="inlineStr">
+      <c r="B97" s="15" t="inlineStr">
         <is>
           <t>Minneapolis, MN; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="C97" s="14" t="inlineStr">
+      <c r="C97" s="15" t="inlineStr">
         <is>
           <t>Minneapolis, MN; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D97" s="16" t="inlineStr">
+      <c r="D97" s="14" t="inlineStr">
         <is>
           <t>Berlin; Ingested — 58 abstracts (Fable)</t>
         </is>
@@ -2725,17 +2764,17 @@
       <c r="A98" s="11" t="n">
         <v>2012</v>
       </c>
-      <c r="B98" s="16" t="inlineStr">
+      <c r="B98" s="14" t="inlineStr">
         <is>
           <t>Vancouver, BC; Ingested</t>
         </is>
       </c>
-      <c r="C98" s="16" t="inlineStr">
+      <c r="C98" s="14" t="inlineStr">
         <is>
           <t>Vancouver, BC (65); Ingested</t>
         </is>
       </c>
-      <c r="D98" s="14" t="inlineStr">
+      <c r="D98" s="15" t="inlineStr">
         <is>
           <t>Milan; Hardcopy — Cat has hardcopy</t>
         </is>
@@ -2751,17 +2790,17 @@
       <c r="A99" s="11" t="n">
         <v>2013</v>
       </c>
-      <c r="B99" s="14" t="inlineStr">
+      <c r="B99" s="15" t="inlineStr">
         <is>
           <t>Albuquerque, NM; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="C99" s="14" t="inlineStr">
+      <c r="C99" s="15" t="inlineStr">
         <is>
           <t>Albuquerque, NM; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D99" s="16" t="inlineStr">
+      <c r="D99" s="14" t="inlineStr">
         <is>
           <t>Plymouth; Ingested — 93 abstracts (Fable)</t>
         </is>
@@ -2773,17 +2812,17 @@
       <c r="A100" s="11" t="n">
         <v>2014</v>
       </c>
-      <c r="B100" s="14" t="inlineStr">
+      <c r="B100" s="15" t="inlineStr">
         <is>
           <t>Chattanooga, TN; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="C100" s="14" t="inlineStr">
+      <c r="C100" s="15" t="inlineStr">
         <is>
           <t>Chattanooga, TN; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D100" s="16" t="inlineStr">
+      <c r="D100" s="14" t="inlineStr">
         <is>
           <t>Leeuwarden; Ingested — 61 abstracts (Fable)</t>
         </is>
@@ -2803,12 +2842,12 @@
       <c r="A101" s="11" t="n">
         <v>2015</v>
       </c>
-      <c r="B101" s="16" t="inlineStr">
+      <c r="B101" s="14" t="inlineStr">
         <is>
           <t>Reno, NV; Ingested</t>
         </is>
       </c>
-      <c r="C101" s="16" t="inlineStr">
+      <c r="C101" s="14" t="inlineStr">
         <is>
           <t>Reno, NV (123); Ingested</t>
         </is>
@@ -2825,17 +2864,17 @@
       <c r="A102" s="11" t="n">
         <v>2016</v>
       </c>
-      <c r="B102" s="16" t="inlineStr">
+      <c r="B102" s="14" t="inlineStr">
         <is>
           <t>New Orleans, LA; Ingested</t>
         </is>
       </c>
-      <c r="C102" s="16" t="inlineStr">
+      <c r="C102" s="14" t="inlineStr">
         <is>
           <t>New Orleans, LA (240); Ingested</t>
         </is>
       </c>
-      <c r="D102" s="16" t="inlineStr">
+      <c r="D102" s="14" t="inlineStr">
         <is>
           <t>Bristol; Ingested — 93 abstracts (Fable)</t>
         </is>
@@ -2861,7 +2900,7 @@
           <t>Austin, TX; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
       </c>
-      <c r="D103" s="16" t="inlineStr">
+      <c r="D103" s="14" t="inlineStr">
         <is>
           <t>Amsterdam; Ingested — 62 talks, programme/no bodies (Fable)</t>
         </is>
@@ -2873,17 +2912,17 @@
       <c r="A104" s="11" t="n">
         <v>2018</v>
       </c>
-      <c r="B104" s="14" t="inlineStr">
+      <c r="B104" s="15" t="inlineStr">
         <is>
           <t>Rochester, NY; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="C104" s="14" t="inlineStr">
+      <c r="C104" s="15" t="inlineStr">
         <is>
           <t>Rochester, NY; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D104" s="16" t="inlineStr">
+      <c r="D104" s="14" t="inlineStr">
         <is>
           <t>Peniche; Ingested — 75 abstracts (Fable)</t>
         </is>
@@ -2893,7 +2932,7 @@
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
       </c>
-      <c r="F104" s="16" t="inlineStr">
+      <c r="F104" s="14" t="inlineStr">
         <is>
           <t>Joao Pessoa; Ingested</t>
         </is>
@@ -2913,7 +2952,7 @@
           <t>Snowbird, UT; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
       </c>
-      <c r="D105" s="16" t="inlineStr">
+      <c r="D105" s="14" t="inlineStr">
         <is>
           <t>Rende; Ingested — 136 abstracts (Fable)</t>
         </is>
@@ -2925,12 +2964,12 @@
       <c r="A106" s="11" t="n">
         <v>2020</v>
       </c>
-      <c r="B106" s="14" t="inlineStr">
+      <c r="B106" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="C106" s="14" t="inlineStr">
+      <c r="C106" s="15" t="inlineStr">
         <is>
           <t>?; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
@@ -2953,12 +2992,12 @@
       </c>
       <c r="B107" s="19" t="inlineStr">
         <is>
-          <t>Phoenix, AZ; Schedule — programme ingested (no abstract bodies)</t>
+          <t>Phoenix, AZ; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
       <c r="C107" s="19" t="inlineStr">
         <is>
-          <t>Phoenix, AZ (46); Schedule — programme ingested (no abstract bodies)</t>
+          <t>Phoenix, AZ (46); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
       <c r="D107" s="18" t="inlineStr">
@@ -2975,12 +3014,12 @@
       </c>
       <c r="B108" s="19" t="inlineStr">
         <is>
-          <t>Spokane, WA; Schedule — programme ingested (no abstract bodies)</t>
+          <t>Spokane, WA; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
       <c r="C108" s="19" t="inlineStr">
         <is>
-          <t>Spokane, WA (69); Schedule — programme ingested (no abstract bodies)</t>
+          <t>Spokane, WA (69); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
       <c r="D108" s="19" t="inlineStr">
@@ -3005,15 +3044,15 @@
       </c>
       <c r="B109" s="19" t="inlineStr">
         <is>
-          <t>Norfolk, VA; Schedule — programme ingested (no abstract bodies)</t>
+          <t>Norfolk, VA; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
       <c r="C109" s="19" t="inlineStr">
         <is>
-          <t>Norfolk, VA (87); Schedule — programme ingested (no abstract bodies)</t>
-        </is>
-      </c>
-      <c r="D109" s="16" t="inlineStr">
+          <t>Norfolk, VA (87); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
+        </is>
+      </c>
+      <c r="D109" s="14" t="inlineStr">
         <is>
           <t>Brighton; Ingested — oral 64 + poster 34 = 98 abstracts (Fable)</t>
         </is>
@@ -3027,12 +3066,12 @@
       </c>
       <c r="B110" s="19" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA; Schedule — programme ingested (no abstract bodies)</t>
+          <t>Pittsburgh, PA; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
       <c r="C110" s="19" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA (97); Schedule — programme ingested (no abstract bodies)</t>
+          <t>Pittsburgh, PA (97); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
       <c r="D110" s="17" t="inlineStr">
@@ -3053,12 +3092,12 @@
       </c>
       <c r="B111" s="19" t="inlineStr">
         <is>
-          <t>St. Paul, MN; Schedule — programme ingested (no abstract bodies)</t>
+          <t>St. Paul, MN; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
       <c r="C111" s="19" t="inlineStr">
         <is>
-          <t>St. Paul, MN (68); Schedule — programme ingested (no abstract bodies)</t>
+          <t>St. Paul, MN (68); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
       <c r="D111" s="17" t="inlineStr">
@@ -3093,7 +3132,7 @@
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
       </c>
-      <c r="F112" s="16" t="inlineStr">
+      <c r="F112" s="14" t="inlineStr">
         <is>
           <t>Colombo; Ingested</t>
         </is>
@@ -3110,7 +3149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3156,6 +3195,11 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
+          <t>EEA</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
@@ -3165,7 +3209,7 @@
         <v>1992</v>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -3180,6 +3224,9 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3188,7 +3235,7 @@
         <v>1993</v>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -3203,6 +3250,9 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3211,7 +3261,7 @@
         <v>1994</v>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -3226,6 +3276,9 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3234,7 +3287,7 @@
         <v>1995</v>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -3249,6 +3302,9 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3257,7 +3313,7 @@
         <v>1996</v>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -3272,6 +3328,9 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3280,7 +3339,7 @@
         <v>1997</v>
       </c>
       <c r="B9" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -3295,6 +3354,9 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3303,7 +3365,7 @@
         <v>1998</v>
       </c>
       <c r="B10" t="n">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -3318,6 +3380,9 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3326,7 +3391,7 @@
         <v>1999</v>
       </c>
       <c r="B11" t="n">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
@@ -3341,6 +3406,9 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3349,7 +3417,7 @@
         <v>2000</v>
       </c>
       <c r="B12" t="n">
-        <v>59</v>
+        <v>134</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
@@ -3364,6 +3432,9 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3372,7 +3443,7 @@
         <v>2001</v>
       </c>
       <c r="B13" t="n">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
@@ -3387,6 +3458,9 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3395,7 +3469,7 @@
         <v>2002</v>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
@@ -3410,6 +3484,9 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3418,7 +3495,7 @@
         <v>2003</v>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
@@ -3433,6 +3510,9 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3441,7 +3521,7 @@
         <v>2004</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
@@ -3456,6 +3536,9 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
+        <v>55</v>
+      </c>
+      <c r="H16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3464,7 +3547,7 @@
         <v>2005</v>
       </c>
       <c r="B17" t="n">
-        <v>81</v>
+        <v>158</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
@@ -3479,6 +3562,9 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3504,6 +3590,9 @@
       <c r="G18" t="n">
         <v>0</v>
       </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -3527,6 +3616,9 @@
       <c r="G19" t="n">
         <v>0</v>
       </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3550,6 +3642,9 @@
       <c r="G20" t="n">
         <v>0</v>
       </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -3573,6 +3668,9 @@
       <c r="G21" t="n">
         <v>0</v>
       </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -3596,6 +3694,9 @@
       <c r="G22" t="n">
         <v>0</v>
       </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -3617,6 +3718,9 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
+        <v>58</v>
+      </c>
+      <c r="H23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3642,6 +3746,9 @@
       <c r="G24" t="n">
         <v>0</v>
       </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -3663,6 +3770,9 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
+        <v>93</v>
+      </c>
+      <c r="H25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3686,6 +3796,9 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
+        <v>61</v>
+      </c>
+      <c r="H26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3711,6 +3824,9 @@
       <c r="G27" t="n">
         <v>0</v>
       </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3732,6 +3848,9 @@
         <v>27</v>
       </c>
       <c r="G28" t="n">
+        <v>93</v>
+      </c>
+      <c r="H28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3755,6 +3874,9 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
+        <v>62</v>
+      </c>
+      <c r="H29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3778,6 +3900,9 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
+        <v>75</v>
+      </c>
+      <c r="H30" t="n">
         <v>427</v>
       </c>
     </row>
@@ -3801,6 +3926,9 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
+        <v>136</v>
+      </c>
+      <c r="H31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3826,6 +3954,9 @@
       <c r="G32" t="n">
         <v>0</v>
       </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3849,6 +3980,9 @@
       <c r="G33" t="n">
         <v>0</v>
       </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -3870,6 +4004,9 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
         <v>89</v>
       </c>
     </row>
@@ -3893,6 +4030,9 @@
         <v>0</v>
       </c>
       <c r="G35" t="n">
+        <v>98</v>
+      </c>
+      <c r="H35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3918,6 +4058,9 @@
       <c r="G36" t="n">
         <v>0</v>
       </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3941,6 +4084,9 @@
       <c r="G37" t="n">
         <v>0</v>
       </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3962,6 +4108,9 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
         <v>1001</v>
       </c>
     </row>
@@ -3972,7 +4121,7 @@
         </is>
       </c>
       <c r="B39" s="1" t="n">
-        <v>1654</v>
+        <v>2346</v>
       </c>
       <c r="C39" s="1" t="n">
         <v>1984</v>
@@ -3987,6 +4136,9 @@
         <v>99</v>
       </c>
       <c r="G39" s="1" t="n">
+        <v>731</v>
+      </c>
+      <c r="H39" s="1" t="n">
         <v>1517</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(conf-abstracts): coverage matrix after Fable 2005/2016 + 2026 schedule
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -2871,7 +2871,7 @@
       </c>
       <c r="C102" s="14" t="inlineStr">
         <is>
-          <t>New Orleans, LA (240); Ingested</t>
+          <t>New Orleans, LA (251); Ingested</t>
         </is>
       </c>
       <c r="D102" s="14" t="inlineStr">
@@ -3112,14 +3112,14 @@
       <c r="A112" s="11" t="n">
         <v>2026</v>
       </c>
-      <c r="B112" s="18" t="inlineStr">
-        <is>
-          <t>New Orleans, LA; Programme — schedule-only programme (OCR text layer OK, not yet parsed) — abstract book needed</t>
-        </is>
-      </c>
-      <c r="C112" s="18" t="inlineStr">
-        <is>
-          <t>New Orleans, LA; Programme — schedule-only programme (OCR text layer OK, not yet parsed) — abstract book needed</t>
+      <c r="B112" s="19" t="inlineStr">
+        <is>
+          <t>New Orleans, LA; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
+        </is>
+      </c>
+      <c r="C112" s="19" t="inlineStr">
+        <is>
+          <t>New Orleans, LA (61); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
       <c r="D112" s="17" t="inlineStr">
@@ -3553,10 +3553,10 @@
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -3573,7 +3573,7 @@
         <v>2006</v>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
@@ -3599,7 +3599,7 @@
         <v>2007</v>
       </c>
       <c r="B19" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C19" t="n">
         <v>427</v>
@@ -3625,7 +3625,7 @@
         <v>2008</v>
       </c>
       <c r="B20" t="n">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C20" t="n">
         <v>215</v>
@@ -3651,7 +3651,7 @@
         <v>2009</v>
       </c>
       <c r="B21" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C21" t="n">
         <v>454</v>
@@ -3677,7 +3677,7 @@
         <v>2010</v>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
@@ -3703,7 +3703,7 @@
         <v>2011</v>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
@@ -3729,7 +3729,7 @@
         <v>2012</v>
       </c>
       <c r="B24" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
@@ -3755,7 +3755,7 @@
         <v>2013</v>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C25" t="n">
         <v>0</v>
@@ -3781,7 +3781,7 @@
         <v>2014</v>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
         <v>0</v>
@@ -3807,7 +3807,7 @@
         <v>2015</v>
       </c>
       <c r="B27" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C27" t="n">
         <v>285</v>
@@ -3833,19 +3833,19 @@
         <v>2016</v>
       </c>
       <c r="B28" t="n">
-        <v>241</v>
+        <v>162</v>
       </c>
       <c r="C28" t="n">
-        <v>375</v>
+        <v>137</v>
       </c>
       <c r="D28" t="n">
-        <v>204</v>
+        <v>39</v>
       </c>
       <c r="E28" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F28" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="G28" t="n">
         <v>93</v>
@@ -3859,7 +3859,7 @@
         <v>2017</v>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
@@ -3885,7 +3885,7 @@
         <v>2018</v>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
@@ -3911,7 +3911,7 @@
         <v>2019</v>
       </c>
       <c r="B31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C31" t="n">
         <v>0</v>
@@ -4093,19 +4093,19 @@
         <v>2026</v>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -4121,19 +4121,19 @@
         </is>
       </c>
       <c r="B39" s="1" t="n">
-        <v>2346</v>
+        <v>2282</v>
       </c>
       <c r="C39" s="1" t="n">
-        <v>1984</v>
+        <v>1767</v>
       </c>
       <c r="D39" s="1" t="n">
-        <v>998</v>
+        <v>845</v>
       </c>
       <c r="E39" s="1" t="n">
-        <v>228</v>
+        <v>329</v>
       </c>
       <c r="F39" s="1" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G39" s="1" t="n">
         <v>731</v>

</xml_diff>

<commit_message>
docs(conf-abstracts): dashboard after Ollama society backfill (3,507 JMIH/ASIH records tagged)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -3342,10 +3342,10 @@
         <v>68</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>345</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -3368,16 +3368,16 @@
         <v>63</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -3394,16 +3394,16 @@
         <v>78</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>237</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -3420,16 +3420,16 @@
         <v>134</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>213</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -3446,10 +3446,10 @@
         <v>84</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>199</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -3533,7 +3533,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
         <v>55</v>
@@ -3547,19 +3547,19 @@
         <v>2005</v>
       </c>
       <c r="B17" t="n">
-        <v>158</v>
+        <v>192</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>448</v>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>345</v>
       </c>
       <c r="E17" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -3628,10 +3628,10 @@
         <v>193</v>
       </c>
       <c r="C20" t="n">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="D20" t="n">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="E20" t="n">
         <v>27</v>
@@ -3654,7 +3654,7 @@
         <v>149</v>
       </c>
       <c r="C21" t="n">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="D21" t="n">
         <v>215</v>
@@ -3663,7 +3663,7 @@
         <v>44</v>
       </c>
       <c r="F21" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -3732,16 +3732,16 @@
         <v>65</v>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>132</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>239</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -3810,7 +3810,7 @@
         <v>123</v>
       </c>
       <c r="C27" t="n">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="D27" t="n">
         <v>130</v>
@@ -3833,19 +3833,19 @@
         <v>2016</v>
       </c>
       <c r="B28" t="n">
-        <v>162</v>
+        <v>245</v>
       </c>
       <c r="C28" t="n">
-        <v>137</v>
+        <v>443</v>
       </c>
       <c r="D28" t="n">
-        <v>39</v>
+        <v>258</v>
       </c>
       <c r="E28" t="n">
         <v>97</v>
       </c>
       <c r="F28" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G28" t="n">
         <v>93</v>
@@ -4121,19 +4121,19 @@
         </is>
       </c>
       <c r="B39" s="1" t="n">
-        <v>2282</v>
+        <v>2399</v>
       </c>
       <c r="C39" s="1" t="n">
-        <v>1767</v>
+        <v>3731</v>
       </c>
       <c r="D39" s="1" t="n">
-        <v>845</v>
+        <v>2088</v>
       </c>
       <c r="E39" s="1" t="n">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="F39" s="1" t="n">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="G39" s="1" t="n">
         <v>731</v>

</xml_diff>

<commit_message>
docs(conf-abstracts): dashboard after society backfill rerun
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -3345,7 +3345,7 @@
         <v>345</v>
       </c>
       <c r="D9" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -3397,7 +3397,7 @@
         <v>237</v>
       </c>
       <c r="D11" t="n">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -3420,10 +3420,10 @@
         <v>134</v>
       </c>
       <c r="C12" t="n">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D12" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
         <v>199</v>
       </c>
       <c r="D13" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -3550,10 +3550,10 @@
         <v>192</v>
       </c>
       <c r="C17" t="n">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D17" t="n">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E17" t="n">
         <v>36</v>
@@ -3839,7 +3839,7 @@
         <v>443</v>
       </c>
       <c r="D28" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E28" t="n">
         <v>97</v>
@@ -4124,10 +4124,10 @@
         <v>2399</v>
       </c>
       <c r="C39" s="1" t="n">
-        <v>3731</v>
+        <v>3735</v>
       </c>
       <c r="D39" s="1" t="n">
-        <v>2088</v>
+        <v>2094</v>
       </c>
       <c r="E39" s="1" t="n">
         <v>334</v>

</xml_diff>

<commit_message>
data(conf-abstracts): JMIH 2015 via Fable + society backfill; matrix and exports refreshed
DB of record 12,432 abstracts / 4,956 elasmo. 2015 Reno now Ingested (587
abstracts, 125 AES). 198 records remain society-unresolved: 174 regex-era
parse stubs (flagged needs_review) and 24 clean Fable records the local LLM
could not place.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -2849,7 +2849,7 @@
       </c>
       <c r="C101" s="14" t="inlineStr">
         <is>
-          <t>Reno, NV (123); Ingested</t>
+          <t>Reno, NV (128); Ingested</t>
         </is>
       </c>
       <c r="D101" s="18" t="inlineStr">
@@ -3550,10 +3550,10 @@
         <v>192</v>
       </c>
       <c r="C17" t="n">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D17" t="n">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E17" t="n">
         <v>36</v>
@@ -3807,19 +3807,19 @@
         <v>2015</v>
       </c>
       <c r="B27" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C27" t="n">
-        <v>288</v>
+        <v>310</v>
       </c>
       <c r="D27" t="n">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -3836,10 +3836,10 @@
         <v>245</v>
       </c>
       <c r="C28" t="n">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="D28" t="n">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E28" t="n">
         <v>97</v>
@@ -4121,19 +4121,19 @@
         </is>
       </c>
       <c r="B39" s="1" t="n">
-        <v>2399</v>
+        <v>2401</v>
       </c>
       <c r="C39" s="1" t="n">
-        <v>3735</v>
+        <v>3756</v>
       </c>
       <c r="D39" s="1" t="n">
-        <v>2094</v>
+        <v>2108</v>
       </c>
       <c r="E39" s="1" t="n">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="F39" s="1" t="n">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="G39" s="1" t="n">
         <v>731</v>

</xml_diff>

<commit_message>
data(conf-abstracts): EEA 2024 Thessaloniki abstract book received clean from Cat
111pp, 175k chars, extracts fine (the August copy was corrupt). Filed as
Conferences/2024/2024_EEA_AbstractBook.pdf and queued for Fable as 3 chunks
(worklist 143-145) — blocked on credits. Matrix: 2024 Digital, 2025 Programme
(Cat's new Rotterdam file is the 7-page agenda, byte-identical to the copy
already held; the Rotterdam abstract book is still corrupt and outstanding).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -121,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,6 +158,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1157,7 +1160,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>- EEA 2010-2026 from Cat Gordon (Shark Trust); pre-2010 in Ali's archive. EEA 2004-2019 + 2023 ingested via Fable (731 abstracts, 2026-08-14) and merged into the main DB 2026-08-25; 2024/2025 PDFs corrupt (await clean copies from Cat). SI2022 Valencia schedule ingested.</t>
+          <t>- EEA 2010-2026 from Cat Gordon (Shark Trust); pre-2010 in Ali's archive. EEA 2004-2019 + 2023 ingested via Fable (731 abstracts, 2026-08-14) and merged into the main DB 2026-08-25; 2024 abstract book received clean 2026-08-27 (queued for extraction); 2025 abstract book still corrupt — working copy needed from Cat. SI2022 Valencia schedule ingested.</t>
         </is>
       </c>
     </row>
@@ -3074,9 +3077,9 @@
           <t>Pittsburgh, PA (97); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="D110" s="17" t="inlineStr">
-        <is>
-          <t>Thessaloniki; Pending — PDF corrupt — need clean copy from Cat</t>
+      <c r="D110" s="20" t="inlineStr">
+        <is>
+          <t>Thessaloniki; Digital — clean abstract book received from Cat 2026-08-27 — queued for extraction</t>
         </is>
       </c>
       <c r="E110" s="17" t="inlineStr">
@@ -3100,9 +3103,9 @@
           <t>St. Paul, MN (68); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="D111" s="17" t="inlineStr">
-        <is>
-          <t>Rotterdam; Pending — PDF corrupt — need clean copy from Cat</t>
+      <c r="D111" s="18" t="inlineStr">
+        <is>
+          <t>Rotterdam; Programme — programme held; abstract book still corrupt — working copy needed from Cat</t>
         </is>
       </c>
       <c r="E111" s="13" t="inlineStr"/>
@@ -3156,7 +3159,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Conference abstract coverage — dashboard</t>
         </is>

</xml_diff>

<commit_message>
data(conf-abstracts): EEA 2002 Cardiff + full SI2022 Valencia abstract books from Cat
- 2002 Cardiff: Word booklet (6th EEA conference) converted to PDF, born-digital
  text, 46pp — queued as 1 Fable chunk. Original .doc kept alongside.
- SI2022 Valencia: the real 111pp abstract book (the earlier file was the
  schedule) — queued as 4 chunks; SI added to the Fable scope for 2022 only.
- Matrix reflects Cat 2026-08-27: she holds 2010/2012/2015/2017 hardcopies but
  has no scanning capacity, so those are sought digitally from the host groups
  (IEG, GRIS, APECE, NEV); Ali Hood is searching her paperwork for 2003-2009;
  1997-2001 (conferences 1-5) have no known source. Host group per year recorded.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -151,6 +151,9 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -158,9 +161,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1160,7 +1160,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>- EEA 2010-2026 from Cat Gordon (Shark Trust); pre-2010 in Ali's archive. EEA 2004-2019 + 2023 ingested via Fable (731 abstracts, 2026-08-14) and merged into the main DB 2026-08-25; 2024 abstract book received clean 2026-08-27 (queued for extraction); 2025 abstract book still corrupt — working copy needed from Cat. SI2022 Valencia schedule ingested.</t>
+          <t>- EEA from Cat Gordon (Shark Trust). 2004-2019 + 2023 ingested via Fable and merged 2026-08-25. Received 2026-08-27: 2002 Cardiff booklet, a clean 2024 Thessaloniki book, and the full SI2022 Valencia abstract book (all queued for extraction). 2025 Rotterdam abstract book is still a corrupt file. Cat holds hardcopies of 2010/2012/2015/2017 but has no scanning capacity, so those are being sought digitally from the host groups; Ali Hood is searching her paperwork for 2003-2009. EEA began in 1997 (2002 Cardiff was the 6th).</t>
         </is>
       </c>
     </row>
@@ -2443,9 +2443,9 @@
           <t>Seattle, WA (68); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
-      <c r="D83" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D83" s="12" t="inlineStr">
+        <is>
+          <t>?; Missing — EEA conferences 1-5, no known source</t>
         </is>
       </c>
       <c r="E83" s="13" t="inlineStr"/>
@@ -2465,9 +2465,9 @@
           <t>Guelph, ON (63); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
-      <c r="D84" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D84" s="12" t="inlineStr">
+        <is>
+          <t>?; Missing — EEA conferences 1-5, no known source</t>
         </is>
       </c>
       <c r="E84" s="13" t="inlineStr"/>
@@ -2487,9 +2487,9 @@
           <t>University Park, PA (78); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
-      <c r="D85" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D85" s="12" t="inlineStr">
+        <is>
+          <t>?; Missing — EEA conferences 1-5, no known source</t>
         </is>
       </c>
       <c r="E85" s="13" t="inlineStr"/>
@@ -2509,9 +2509,9 @@
           <t>La Paz, Mexico (134); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
-      <c r="D86" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D86" s="12" t="inlineStr">
+        <is>
+          <t>?; Missing — EEA conferences 1-5, no known source</t>
         </is>
       </c>
       <c r="E86" s="13" t="inlineStr"/>
@@ -2531,9 +2531,9 @@
           <t>University Park, PA (84); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
-      <c r="D87" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D87" s="12" t="inlineStr">
+        <is>
+          <t>?; Missing — EEA conferences 1-5, no known source</t>
         </is>
       </c>
       <c r="E87" s="13" t="inlineStr"/>
@@ -2553,9 +2553,9 @@
           <t>Kansas City, MO (27); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
-      <c r="D88" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D88" s="17" t="inlineStr">
+        <is>
+          <t>Cardiff; Digital — abstract booklet (Word) from Cat 2026-08-27 — queued for extraction</t>
         </is>
       </c>
       <c r="E88" s="13" t="inlineStr"/>
@@ -2575,9 +2575,9 @@
           <t>Manaus, Brazil (82); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
-      <c r="D89" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D89" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E89" s="13" t="inlineStr"/>
@@ -2619,9 +2619,9 @@
           <t>Tampa, FL (158); Ingested — AES abstracts from elasmo.org (full bodies)</t>
         </is>
       </c>
-      <c r="D91" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D91" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E91" s="13" t="inlineStr"/>
@@ -2641,9 +2641,9 @@
           <t>New Orleans, LA; Hardcopy — Carylanne has hardcopy (1992-2024) — get abstract book</t>
         </is>
       </c>
-      <c r="D92" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D92" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E92" s="13" t="inlineStr"/>
@@ -2663,9 +2663,9 @@
           <t>St. Louis, MO (155); Ingested</t>
         </is>
       </c>
-      <c r="D93" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D93" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E93" s="13" t="inlineStr"/>
@@ -2685,9 +2685,9 @@
           <t>Montreal, PQ (193); Ingested</t>
         </is>
       </c>
-      <c r="D94" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D94" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E94" s="13" t="inlineStr"/>
@@ -2707,9 +2707,9 @@
           <t>Portland, OR (149); Ingested</t>
         </is>
       </c>
-      <c r="D95" s="15" t="inlineStr">
-        <is>
-          <t>?; Hardcopy — Ali's archive (back mid-Aug)</t>
+      <c r="D95" s="18" t="inlineStr">
+        <is>
+          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E95" s="13" t="inlineStr"/>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="D96" s="15" t="inlineStr">
         <is>
-          <t>Galway; Hardcopy — Cat has hardcopy</t>
+          <t>Galway; Hardcopy — Cat has hardcopy but no scanning capacity — digital needed from IEG (Ireland)</t>
         </is>
       </c>
       <c r="E96" s="13" t="inlineStr"/>
@@ -2779,10 +2779,10 @@
       </c>
       <c r="D98" s="15" t="inlineStr">
         <is>
-          <t>Milan; Hardcopy — Cat has hardcopy</t>
-        </is>
-      </c>
-      <c r="E98" s="17" t="inlineStr">
+          <t>Milan; Hardcopy — Cat has hardcopy but no scanning capacity — digital needed from GRIS (Italy)</t>
+        </is>
+      </c>
+      <c r="E98" s="18" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -2830,7 +2830,7 @@
           <t>Leeuwarden; Ingested — 61 abstracts (Fable)</t>
         </is>
       </c>
-      <c r="E100" s="17" t="inlineStr">
+      <c r="E100" s="18" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -2855,9 +2855,9 @@
           <t>Reno, NV (128); Ingested</t>
         </is>
       </c>
-      <c r="D101" s="18" t="inlineStr">
-        <is>
-          <t>Peniche; Programme — 2-page programme only (0 abstracts) — abstract book needed</t>
+      <c r="D101" s="19" t="inlineStr">
+        <is>
+          <t>Peniche; Programme — 2-page programme only; Cat has hardcopy but no scanning capacity — abstract book needed from APECE (Portugal)</t>
         </is>
       </c>
       <c r="E101" s="13" t="inlineStr"/>
@@ -2882,7 +2882,7 @@
           <t>Bristol; Ingested — 93 abstracts (Fable)</t>
         </is>
       </c>
-      <c r="E102" s="17" t="inlineStr">
+      <c r="E102" s="18" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -2893,19 +2893,19 @@
       <c r="A103" s="11" t="n">
         <v>2017</v>
       </c>
-      <c r="B103" s="18" t="inlineStr">
+      <c r="B103" s="19" t="inlineStr">
         <is>
           <t>Austin, TX; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
       </c>
-      <c r="C103" s="18" t="inlineStr">
+      <c r="C103" s="19" t="inlineStr">
         <is>
           <t>Austin, TX; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
       </c>
-      <c r="D103" s="14" t="inlineStr">
-        <is>
-          <t>Amsterdam; Ingested — 62 talks, programme/no bodies (Fable)</t>
+      <c r="D103" s="20" t="inlineStr">
+        <is>
+          <t>Amsterdam; Schedule — 62 talks ingested, NO abstract bodies; Cat has hardcopy but no scanning capacity — abstract book needed from NEV</t>
         </is>
       </c>
       <c r="E103" s="13" t="inlineStr"/>
@@ -2930,7 +2930,7 @@
           <t>Peniche; Ingested — 75 abstracts (Fable)</t>
         </is>
       </c>
-      <c r="E104" s="17" t="inlineStr">
+      <c r="E104" s="18" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -2945,12 +2945,12 @@
       <c r="A105" s="11" t="n">
         <v>2019</v>
       </c>
-      <c r="B105" s="18" t="inlineStr">
+      <c r="B105" s="19" t="inlineStr">
         <is>
           <t>Snowbird, UT; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
       </c>
-      <c r="C105" s="18" t="inlineStr">
+      <c r="C105" s="19" t="inlineStr">
         <is>
           <t>Snowbird, UT; Programme — grid programme only — abstract book needed (Carylanne)</t>
         </is>
@@ -2982,7 +2982,7 @@
           <t>online (covid); Missing — covid/online — find</t>
         </is>
       </c>
-      <c r="E106" s="17" t="inlineStr">
+      <c r="E106" s="18" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -2993,19 +2993,19 @@
       <c r="A107" s="11" t="n">
         <v>2021</v>
       </c>
-      <c r="B107" s="19" t="inlineStr">
+      <c r="B107" s="20" t="inlineStr">
         <is>
           <t>Phoenix, AZ; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="C107" s="19" t="inlineStr">
+      <c r="C107" s="20" t="inlineStr">
         <is>
           <t>Phoenix, AZ (46); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="D107" s="18" t="inlineStr">
-        <is>
-          <t>Leiden; Programme — only programme held — abstract book needed</t>
+      <c r="D107" s="19" t="inlineStr">
+        <is>
+          <t>Leiden; Programme — programme only — abstract book needed from NEV</t>
         </is>
       </c>
       <c r="E107" s="13" t="inlineStr"/>
@@ -3015,29 +3015,29 @@
       <c r="A108" s="11" t="n">
         <v>2022</v>
       </c>
-      <c r="B108" s="19" t="inlineStr">
+      <c r="B108" s="20" t="inlineStr">
         <is>
           <t>Spokane, WA; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="C108" s="19" t="inlineStr">
+      <c r="C108" s="20" t="inlineStr">
         <is>
           <t>Spokane, WA (69); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="D108" s="19" t="inlineStr">
-        <is>
-          <t>Valencia (=SI2022); Schedule — covered via SI2022 (schedule)</t>
-        </is>
-      </c>
-      <c r="E108" s="17" t="inlineStr">
+      <c r="D108" s="17" t="inlineStr">
+        <is>
+          <t>Valencia (=SI2022); Digital — full SI2022 abstract book from Cat 2026-08-27 — queued for extraction</t>
+        </is>
+      </c>
+      <c r="E108" s="18" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
       </c>
-      <c r="F108" s="19" t="inlineStr">
-        <is>
-          <t>Valencia; Schedule — programme ingested (no bodies)</t>
+      <c r="F108" s="17" t="inlineStr">
+        <is>
+          <t>Valencia; Digital — full abstract book received 2026-08-27 — queued (schedule already ingested)</t>
         </is>
       </c>
     </row>
@@ -3045,12 +3045,12 @@
       <c r="A109" s="11" t="n">
         <v>2023</v>
       </c>
-      <c r="B109" s="19" t="inlineStr">
+      <c r="B109" s="20" t="inlineStr">
         <is>
           <t>Norfolk, VA; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="C109" s="19" t="inlineStr">
+      <c r="C109" s="20" t="inlineStr">
         <is>
           <t>Norfolk, VA (87); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
@@ -3067,22 +3067,22 @@
       <c r="A110" s="11" t="n">
         <v>2024</v>
       </c>
-      <c r="B110" s="19" t="inlineStr">
+      <c r="B110" s="20" t="inlineStr">
         <is>
           <t>Pittsburgh, PA; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="C110" s="19" t="inlineStr">
+      <c r="C110" s="20" t="inlineStr">
         <is>
           <t>Pittsburgh, PA (97); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="D110" s="20" t="inlineStr">
+      <c r="D110" s="17" t="inlineStr">
         <is>
           <t>Thessaloniki; Digital — clean abstract book received from Cat 2026-08-27 — queued for extraction</t>
         </is>
       </c>
-      <c r="E110" s="17" t="inlineStr">
+      <c r="E110" s="18" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>
@@ -3093,19 +3093,19 @@
       <c r="A111" s="11" t="n">
         <v>2025</v>
       </c>
-      <c r="B111" s="19" t="inlineStr">
+      <c r="B111" s="20" t="inlineStr">
         <is>
           <t>St. Paul, MN; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="C111" s="19" t="inlineStr">
+      <c r="C111" s="20" t="inlineStr">
         <is>
           <t>St. Paul, MN (68); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="D111" s="18" t="inlineStr">
-        <is>
-          <t>Rotterdam; Programme — programme held; abstract book still corrupt — working copy needed from Cat</t>
+      <c r="D111" s="19" t="inlineStr">
+        <is>
+          <t>Rotterdam; Programme — programme held; the abstract-book file is corrupt — working copy needed from NEV / Cat</t>
         </is>
       </c>
       <c r="E111" s="13" t="inlineStr"/>
@@ -3115,22 +3115,22 @@
       <c r="A112" s="11" t="n">
         <v>2026</v>
       </c>
-      <c r="B112" s="19" t="inlineStr">
+      <c r="B112" s="20" t="inlineStr">
         <is>
           <t>New Orleans, LA; Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="C112" s="19" t="inlineStr">
+      <c r="C112" s="20" t="inlineStr">
         <is>
           <t>New Orleans, LA (61); Schedule — programme ingested (no abstract bodies) — abstract book needed</t>
         </is>
       </c>
-      <c r="D112" s="17" t="inlineStr">
+      <c r="D112" s="18" t="inlineStr">
         <is>
           <t>online; Pending — will be digital</t>
         </is>
       </c>
-      <c r="E112" s="17" t="inlineStr">
+      <c r="E112" s="18" t="inlineStr">
         <is>
           <t>?; Pending — Brit collating (council approval)</t>
         </is>

</xml_diff>

<commit_message>
docs(conf-abstracts): correct 2025 Rotterdam status; plainer punctuation in matrix notes and board summary
Cat has no Rotterdam abstract book and is unsure one was produced, so the cell
now asks NEV/Irene to confirm rather than asking Cat for a working copy.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -2555,7 +2555,7 @@
       </c>
       <c r="D88" s="17" t="inlineStr">
         <is>
-          <t>Cardiff; Digital — abstract booklet (Word) from Cat 2026-08-27 — queued for extraction</t>
+          <t>Cardiff; Digital — abstract booklet (Word) found by Ali Hood 2026-08-27; queued for extraction</t>
         </is>
       </c>
       <c r="E88" s="13" t="inlineStr"/>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="D96" s="15" t="inlineStr">
         <is>
-          <t>Galway; Hardcopy — Cat has hardcopy but no scanning capacity — digital needed from IEG (Ireland)</t>
+          <t>Galway; Hardcopy — Cat holds a hardcopy but has no scanning capacity; digital copy needed from IEG (Ireland)</t>
         </is>
       </c>
       <c r="E96" s="13" t="inlineStr"/>
@@ -2779,7 +2779,7 @@
       </c>
       <c r="D98" s="15" t="inlineStr">
         <is>
-          <t>Milan; Hardcopy — Cat has hardcopy but no scanning capacity — digital needed from GRIS (Italy)</t>
+          <t>Milan; Hardcopy — Cat holds a hardcopy but has no scanning capacity; digital copy needed from GRIS (Italy)</t>
         </is>
       </c>
       <c r="E98" s="18" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="D101" s="19" t="inlineStr">
         <is>
-          <t>Peniche; Programme — 2-page programme only; Cat has hardcopy but no scanning capacity — abstract book needed from APECE (Portugal)</t>
+          <t>Peniche; Programme — 2-page programme only; Cat holds a hardcopy but has no scanning capacity; abstract book needed from APECE (Portugal)</t>
         </is>
       </c>
       <c r="E101" s="13" t="inlineStr"/>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="D103" s="20" t="inlineStr">
         <is>
-          <t>Amsterdam; Schedule — 62 talks ingested, NO abstract bodies; Cat has hardcopy but no scanning capacity — abstract book needed from NEV</t>
+          <t>Amsterdam; Schedule — 62 talks ingested, NO abstract bodies; Cat holds a hardcopy but has no scanning capacity; abstract book needed from NEV</t>
         </is>
       </c>
       <c r="E103" s="13" t="inlineStr"/>
@@ -3005,7 +3005,7 @@
       </c>
       <c r="D107" s="19" t="inlineStr">
         <is>
-          <t>Leiden; Programme — programme only — abstract book needed from NEV</t>
+          <t>Leiden; Programme — programme only; abstract book needed from NEV</t>
         </is>
       </c>
       <c r="E107" s="13" t="inlineStr"/>
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D108" s="17" t="inlineStr">
         <is>
-          <t>Valencia (=SI2022); Digital — full SI2022 abstract book from Cat 2026-08-27 — queued for extraction</t>
+          <t>Valencia (=SI2022); Digital — full SI2022 abstract book received 2026-08-27; queued for extraction</t>
         </is>
       </c>
       <c r="E108" s="18" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="F108" s="17" t="inlineStr">
         <is>
-          <t>Valencia; Digital — full abstract book received 2026-08-27 — queued (schedule already ingested)</t>
+          <t>Valencia; Digital — full abstract book received 2026-08-27; queued (schedule already ingested)</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="D110" s="17" t="inlineStr">
         <is>
-          <t>Thessaloniki; Digital — clean abstract book received from Cat 2026-08-27 — queued for extraction</t>
+          <t>Thessaloniki; Digital — clean abstract book received from Cat 2026-08-27; queued for extraction</t>
         </is>
       </c>
       <c r="E110" s="18" t="inlineStr">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="D111" s="19" t="inlineStr">
         <is>
-          <t>Rotterdam; Programme — programme held; the abstract-book file is corrupt — working copy needed from NEV / Cat</t>
+          <t>Rotterdam; Programme — agenda only; Cat has no abstract book and is unsure one was produced; NEV/Irene to confirm whether it exists</t>
         </is>
       </c>
       <c r="E111" s="13" t="inlineStr"/>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="D112" s="18" t="inlineStr">
         <is>
-          <t>online; Pending — will be digital</t>
+          <t>online; Pending — will be digital (Shark Trust hosting)</t>
         </is>
       </c>
       <c r="E112" s="18" t="inlineStr">

</xml_diff>

<commit_message>
feat(conf-abstracts): colour ramp ordered by distance from done; early EEA and OCS host cities
Ramp is now strictly Missing < Schedule < Hardcopy < Programme < Pending < OCR
< Digital < Ingested. Digital (book in hand, extraction pending) reads light
green; OCR (abstracts in but from a degraded scan) drops back to yellow;
Schedule (titles, no abstract text) sits just above Missing; Hardcopy and
Programme are adjacent since both mean 'we still need the book'.

Host cities added from the EEA's own meetings page: 2003 San Marino, 2005
Monaco, 2006 Hamburg, 2007 Brest, 2008 Lisbon, 2009 Palma de Majorca, plus 1998
Lisbon from APECE. Meeting numbers there confirm an unbroken annual series from
1997, matching the 2002 Cardiff booklet's '6th'. OCS: 2012 Adelaide, 2018 North
Stradbroke Island, 2024 Geelong.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -56,6 +56,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F0A868"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F6B26B"/>
       </patternFill>
     </fill>
@@ -66,12 +71,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE599"/>
+        <fgColor rgb="00FFD966"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD966"/>
+        <fgColor rgb="00FFE599"/>
       </patternFill>
     </fill>
     <fill>
@@ -82,11 +87,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="006AA84F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D2E9"/>
       </patternFill>
     </fill>
     <fill>
@@ -142,10 +142,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -154,13 +160,7 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>No known source anywhere</t>
+          <t>No known source anywhere.</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -1017,12 +1017,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hardcopy</t>
+          <t>Schedule</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Physical book exists (Carylanne / Cat / Ali), not digitised</t>
+          <t>Programme ingested: titles, authors, presentation type. NO abstract text. Useful, but it isn't abstracts.</t>
         </is>
       </c>
       <c r="C3" s="3" t="n"/>
@@ -1030,12 +1030,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Programme</t>
+          <t>Hardcopy</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Digital PROGRAMME/schedule held, but NOT full abstracts — the abstract book is still needed (see note)</t>
+          <t>A physical book is known to exist (Carylanne, Cat, Ali) but nothing digital. Needs scanning, or a digital copy from the host.</t>
         </is>
       </c>
       <c r="C4" s="4" t="n"/>
@@ -1043,12 +1043,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Digital</t>
+          <t>Programme</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Digital ABSTRACT BOOK held &amp; ingestable, not yet ingested</t>
+          <t>A digital programme is held, but not the abstract book. Same practical need as Hardcopy: get the book.</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
@@ -1056,12 +1056,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>OCR</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Full abstracts ingested but from degraded scans (needs_review) — flatbed re-scan planned</t>
+          <t>A named contact has it or is looking for it, not yet received (EEA: Cat and Ali; OCS: Brit).</t>
         </is>
       </c>
       <c r="C6" s="6" t="n"/>
@@ -1069,12 +1069,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Schedule</t>
+          <t>OCR</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Programme ingested: titles/authors/type, NO abstract bodies</t>
+          <t>Abstracts ingested, but from a degraded scan and flagged needs_review. Still worth re-sourcing a clean copy.</t>
         </is>
       </c>
       <c r="C7" s="7" t="n"/>
@@ -1082,12 +1082,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ingested</t>
+          <t>Digital</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Full abstracts ingested into the DB</t>
+          <t>Abstract book in hand and ingestable. Only extraction remains.</t>
         </is>
       </c>
       <c r="C8" s="8" t="n"/>
@@ -1095,12 +1095,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Ingested</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Available from an external contact, not yet obtained (EEA: Cat; OCS: Brit)</t>
+          <t>Full abstracts ingested into the database.</t>
         </is>
       </c>
       <c r="C9" s="9" t="n"/>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="D83" s="12" t="inlineStr">
         <is>
-          <t>?; Missing — EEA conferences 1-5, no known source</t>
+          <t>?; Missing — 1st EEA; no known abstract source; host city also unknown</t>
         </is>
       </c>
       <c r="E83" s="13" t="inlineStr"/>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>?; Missing — EEA conferences 1-5, no known source</t>
+          <t>Lisbon; Missing — 2nd EEA; no known abstract source</t>
         </is>
       </c>
       <c r="E84" s="13" t="inlineStr"/>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="D85" s="12" t="inlineStr">
         <is>
-          <t>?; Missing — EEA conferences 1-5, no known source</t>
+          <t>?; Missing — 3rd EEA; no known abstract source; host city also unknown</t>
         </is>
       </c>
       <c r="E85" s="13" t="inlineStr"/>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
-          <t>?; Missing — EEA conferences 1-5, no known source</t>
+          <t>?; Missing — 4th EEA; no known abstract source; host city also unknown</t>
         </is>
       </c>
       <c r="E86" s="13" t="inlineStr"/>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="D87" s="12" t="inlineStr">
         <is>
-          <t>?; Missing — EEA conferences 1-5, no known source</t>
+          <t>?; Missing — 5th EEA; no known abstract source; host city also unknown</t>
         </is>
       </c>
       <c r="E87" s="13" t="inlineStr"/>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="D89" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
+          <t>San Marino; Pending — 7th EEA; Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E89" s="13" t="inlineStr"/>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="D91" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
+          <t>Monaco; Pending — 9th EEA; Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E91" s="13" t="inlineStr"/>
@@ -2643,7 +2643,7 @@
       </c>
       <c r="D92" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
+          <t>Hamburg; Pending — 10th EEA; Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E92" s="13" t="inlineStr"/>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="D93" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
+          <t>Brest; Pending — 11th EEA; Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E93" s="13" t="inlineStr"/>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="D94" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
+          <t>Lisbon; Pending — 12th EEA; Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E94" s="13" t="inlineStr"/>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="D95" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Ali Hood searching her paperwork (2026-08-27)</t>
+          <t>Palma de Majorca; Pending — 13th EEA; Ali Hood searching her paperwork (2026-08-27)</t>
         </is>
       </c>
       <c r="E95" s="13" t="inlineStr"/>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="E98" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Brit collating (council approval)</t>
+          <t>Adelaide; Pending — joint with ASFB; Brit Finucci confirming</t>
         </is>
       </c>
       <c r="F98" s="13" t="inlineStr"/>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="E100" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Brit collating (council approval)</t>
+          <t>?; Pending — Brit Finucci collating; year/location to confirm</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="E102" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Brit collating (council approval)</t>
+          <t>?; Pending — Brit Finucci collating; year/location to confirm</t>
         </is>
       </c>
       <c r="F102" s="13" t="inlineStr"/>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="E104" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Brit collating (council approval)</t>
+          <t>North Stradbroke Is.; Pending — Moreton Bay Research Station; Brit Finucci confirming</t>
         </is>
       </c>
       <c r="F104" s="14" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="E106" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Brit collating (council approval)</t>
+          <t>?; Pending — Brit Finucci collating; year/location to confirm</t>
         </is>
       </c>
       <c r="F106" s="13" t="inlineStr"/>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="E108" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Brit collating (council approval)</t>
+          <t>?; Pending — Brit Finucci collating; year/location to confirm</t>
         </is>
       </c>
       <c r="F108" s="17" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="E110" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Brit collating (council approval)</t>
+          <t>Geelong; Pending — Brit Finucci confirming</t>
         </is>
       </c>
       <c r="F110" s="13" t="inlineStr"/>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="E112" s="18" t="inlineStr">
         <is>
-          <t>?; Pending — Brit collating (council approval)</t>
+          <t>?; Pending — Brit Finucci collating; year/location to confirm</t>
         </is>
       </c>
       <c r="F112" s="14" t="inlineStr">

</xml_diff>

<commit_message>
data(conf-abstracts): EEA 2015 Peniche Book of Abstracts found locally; ramp reorder; 2020 unknown
- 2015: Simon's own copy of the 19th EEA Book of Abstracts (99pp, born-digital
  Word, full bodies + 'Presentation type' markers). Filed to Conferences/2015
  and queued as 2 chunks. Stale EEA2015 cache (the 2-page programme, 0
  abstracts) deleted so extraction actually runs.
- Colour ramp: OCR moves between Hardcopy and Programme per Simon, since a
  degraded scan is functionally the same problem as an unscanned hardcopy.
  Order is now Missing < Schedule < Hardcopy < OCR < Programme < Pending <
  Digital < Ingested.
- 2020: we do not know whether a meeting was held. Cat thinks it was online for
  covid but was on maternity leave and is unsure; organiser unknown. The cell
  no longer asserts an online meeting took place.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -56,7 +56,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0A868"/>
+        <fgColor rgb="00ED9C6B"/>
       </patternFill>
     </fill>
     <fill>
@@ -148,16 +148,16 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1043,12 +1043,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Programme</t>
+          <t>OCR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>A digital programme is held, but not the abstract book. Same practical need as Hardcopy: get the book.</t>
+          <t>Abstracts ingested, but from a degraded scan and flagged needs_review. Still worth re-sourcing a clean copy.</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
@@ -1056,12 +1056,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Programme</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>A named contact has it or is looking for it, not yet received (EEA: Cat and Ali; OCS: Brit).</t>
+          <t>A digital programme is held, but not the abstract book. Same practical need as Hardcopy: get the book.</t>
         </is>
       </c>
       <c r="C6" s="6" t="n"/>
@@ -1069,12 +1069,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>OCR</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Abstracts ingested, but from a degraded scan and flagged needs_review. Still worth re-sourcing a clean copy.</t>
+          <t>A named contact has it or is looking for it, not yet received (EEA: Cat and Ali; OCS: Brit).</t>
         </is>
       </c>
       <c r="C7" s="7" t="n"/>
@@ -2855,9 +2855,9 @@
           <t>Reno, NV (128); Ingested</t>
         </is>
       </c>
-      <c r="D101" s="19" t="inlineStr">
-        <is>
-          <t>Peniche; Programme — 2-page programme only; Cat holds a hardcopy but has no scanning capacity; abstract book needed from APECE (Portugal)</t>
+      <c r="D101" s="17" t="inlineStr">
+        <is>
+          <t>Peniche; Digital — 19th EEA Book of Abstracts (99pp, born-digital) held by Simon all along; queued for extraction</t>
         </is>
       </c>
       <c r="E101" s="13" t="inlineStr"/>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>online (covid); Missing — covid/online — find</t>
+          <t>?; Missing — unknown whether a meeting was held: Cat thinks it was online for covid but was on maternity leave and is unsure; organiser unknown; abstracts unknown</t>
         </is>
       </c>
       <c r="E106" s="18" t="inlineStr">

</xml_diff>

<commit_message>
feat(conf-abstracts): preserve human legend edits; add % meetings-ingested chart
The builder regenerates the whole workbook, so wording Simon edited in Legend &
Notes was being silently reverted on the next run. It now harvests the live
sheet's meanings and notes into data/matrix_legend.json before rebuilding and
re-emits those, with code defaults only filling gaps. This run rescued four
edited meanings (Hardcopy, OCR, Pending, Programme) that would otherwise have
been lost. --reset-legend forces code wording. check_coverage_matrix --legend
reports drift.

Dashboard gains a second chart beside the totals: '% of meetings with abstracts
ingested, by society' for AES, EEA, OCS, SI, with a backing table. Denominator
is meetings known to have taken place, not abstracts, so SI reads n/5. Current:
AES 27/44 (61%), EEA 8/30 (27%), OCS 0/8, SI 2/5 (40%).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/conference_coverage_matrix.xlsx
+++ b/database/conference_coverage_matrix.xlsx
@@ -341,6 +341,97 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>% of meetings with abstracts ingested, by society</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$43:$A$46</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$D$43:$D$46</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="100"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% of that society's meetings</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Abstracts over time, by society/series</a:t>
             </a:r>
           </a:p>
@@ -665,12 +756,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>18</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="3600000"/>
+    <ext cx="5760000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -680,6 +771,28 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -977,7 +1090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1035,7 +1148,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A physical book is known to exist (Carylanne, Cat, Ali) but nothing digital. Needs scanning, or a digital copy from the host.</t>
+          <t>Physical book known to exist (Carylanne, Cat, Ali) but nothing digital. Needs scanning, or a digital copy.</t>
         </is>
       </c>
       <c r="C4" s="4" t="n"/>
@@ -1048,7 +1161,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Abstracts ingested, but from a degraded scan and flagged needs_review. Still worth re-sourcing a clean copy.</t>
+          <t>Abstracts ingested, but from a degraded scan and flagged needs_review. Worth re-sourcing a clean copy, ideally digital.</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
@@ -1061,7 +1174,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>A digital programme is held, but not the abstract book. Same practical need as Hardcopy: get the book.</t>
+          <t>Digital programme held, not the abstract book. Per Hardcopy: get the book, ideally digital.</t>
         </is>
       </c>
       <c r="C6" s="6" t="n"/>
@@ -1074,7 +1187,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>A named contact has it or is looking for it, not yet received (EEA: Cat and Ali; OCS: Brit).</t>
+          <t>A named contact has it or is looking for it, not yet received.</t>
         </is>
       </c>
       <c r="C7" s="7" t="n"/>
@@ -1106,80 +1219,70 @@
       <c r="C9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>- 'ASIH/JMIH' = the American joint meeting (ASIH pre-1997, JMIH from 1997). ASIH/JMIH/HL/SSAR/NIA share one source book, collapsed to this column to remove duplicates.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NOTES:</t>
+          <t>- 'AES' (American Elasmobranch Society, founded 1983) kept separate — cell shows elasmo-abstract count where ingested. Pre-1983 = no conference (blank).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>- 'ASIH/JMIH' = the American joint meeting (ASIH pre-1997, JMIH from 1997). ASIH/JMIH/HL/SSAR/NIA share one source book, collapsed to this column to remove duplicates.</t>
+          <t>- Host cities 1916-2025 from github.com/SimonDedman/AESconfLocations; 2026 = New Orleans.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>- 'AES' (American Elasmobranch Society, founded 1983) kept separate — cell shows elasmo-abstract count where ingested. Pre-1983 = no conference (blank).</t>
+          <t>- 'OCR' = degraded 1997-2004 JMIH phone-photo scans (all needs_review); Carylanne's flatbed re-scans would upgrade the non-AES content.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>- Host cities 1916-2025 from github.com/SimonDedman/AESconfLocations; 2026 = New Orleans.</t>
+          <t>- AES 1985-2005: full abstracts harvested from elasmo.org/meetings/abstracts/abst&lt;YYYY&gt;/ (1,305 abstracts, 2026-08-25); JMIH-book copies of the same AES talks were removed. No AES source found for 1983-84 or 2006+ online.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>- 'OCR' = degraded 1997-2004 JMIH phone-photo scans (all needs_review); Carylanne's flatbed re-scans would upgrade the non-AES content.</t>
+          <t>- ASIH/JMIH pre-1992: Carylanne's archive starts 1992 → host city shown but 'Missing'.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>- AES 1985-2005: full abstracts harvested from elasmo.org/meetings/abstracts/abst&lt;YYYY&gt;/ (1,305 abstracts, 2026-08-25); JMIH-book copies of the same AES talks were removed. No AES source found for 1983-84 or 2006+ online.</t>
+          <t>- EEA from Cat Gordon (Shark Trust). 2004-2019 + 2023 ingested via Fable and merged 2026-08-25. Received 2026-08-27: 2002 Cardiff booklet, a clean 2024 Thessaloniki book, and the full SI2022 Valencia abstract book (all queued for extraction). 2025 Rotterdam abstract book is still a corrupt file. Cat holds hardcopies of 2010/2012/2015/2017 but has no scanning capacity, so those are being sought digitally from the host groups; Ali Hood is searching her paperwork for 2003-2009. EEA began in 1997 (2002 Cardiff was the 6th).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>- ASIH/JMIH pre-1992: Carylanne's archive starts 1992 → host city shown but 'Missing'.</t>
+          <t>- OCS (Oceania Chondrichthyan Soc, ~2011+, biennial): Brit Finucci collating, pending council — years/locations TBC.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>- EEA from Cat Gordon (Shark Trust). 2004-2019 + 2023 ingested via Fable and merged 2026-08-25. Received 2026-08-27: 2002 Cardiff booklet, a clean 2024 Thessaloniki book, and the full SI2022 Valencia abstract book (all queued for extraction). 2025 Rotterdam abstract book is still a corrupt file. Cat holds hardcopies of 2010/2012/2015/2017 but has no scanning capacity, so those are being sought digitally from the host groups; Ali Hood is searching her paperwork for 2003-2009. EEA began in 1997 (2002 Cardiff was the 6th).</t>
+          <t>- Blank/unshaded cell = no conference that year for that series.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
-        <is>
-          <t>- OCS (Oceania Chondrichthyan Soc, ~2011+, biennial): Brit Finucci collating, pending council — years/locations TBC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>- Blank/unshaded cell = no conference that year for that series.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
         <is>
           <t>- Per-society counts &amp; trends: see the Dashboard tab.</t>
         </is>
@@ -3152,7 +3255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4145,6 +4248,92 @@
         <v>1517</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>Series</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>Meetings ingested</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>Meetings known</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>% ingested</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AES</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>27</v>
+      </c>
+      <c r="C43" t="n">
+        <v>44</v>
+      </c>
+      <c r="D43" t="n">
+        <v>61.4</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>EEA</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>8</v>
+      </c>
+      <c r="C44" t="n">
+        <v>30</v>
+      </c>
+      <c r="D44" t="n">
+        <v>26.7</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>OCS</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>8</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+      <c r="D46" t="n">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>